<commit_message>
Add Section 32 batch 02 checkpoint
Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
+++ b/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
@@ -3531,27 +3531,47 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr"/>
-      <c r="G52" s="2" t="inlineStr"/>
-      <c r="H52" s="2" t="inlineStr"/>
-      <c r="I52" s="2" t="inlineStr"/>
-      <c r="J52" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>B02-G001; B02-G002</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -3571,27 +3591,47 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr"/>
-      <c r="G53" s="2" t="inlineStr"/>
-      <c r="H53" s="2" t="inlineStr"/>
-      <c r="I53" s="2" t="inlineStr"/>
-      <c r="J53" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>B02-G002</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -3611,27 +3651,47 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr"/>
-      <c r="G54" s="2" t="inlineStr"/>
-      <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="2" t="inlineStr"/>
-      <c r="J54" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>B02-G002</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -3651,27 +3711,47 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr"/>
-      <c r="G55" s="2" t="inlineStr"/>
-      <c r="H55" s="2" t="inlineStr"/>
-      <c r="I55" s="2" t="inlineStr"/>
-      <c r="J55" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>B02-G003; B02-G004</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -3691,27 +3771,47 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr"/>
-      <c r="G56" s="2" t="inlineStr"/>
-      <c r="H56" s="2" t="inlineStr"/>
-      <c r="I56" s="2" t="inlineStr"/>
-      <c r="J56" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>B02-G005</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -3731,27 +3831,47 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr"/>
-      <c r="G57" s="2" t="inlineStr"/>
-      <c r="H57" s="2" t="inlineStr"/>
-      <c r="I57" s="2" t="inlineStr"/>
-      <c r="J57" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>B02-G006</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -3771,27 +3891,47 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr"/>
-      <c r="G58" s="2" t="inlineStr"/>
-      <c r="H58" s="2" t="inlineStr"/>
-      <c r="I58" s="2" t="inlineStr"/>
-      <c r="J58" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>B02-G007</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -3811,27 +3951,47 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F59" s="2" t="inlineStr"/>
-      <c r="G59" s="2" t="inlineStr"/>
-      <c r="H59" s="2" t="inlineStr"/>
-      <c r="I59" s="2" t="inlineStr"/>
-      <c r="J59" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>B02-G007</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -3851,27 +4011,47 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="inlineStr"/>
-      <c r="G60" s="2" t="inlineStr"/>
-      <c r="H60" s="2" t="inlineStr"/>
-      <c r="I60" s="2" t="inlineStr"/>
-      <c r="J60" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>B02-G008; B02-G009</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -3891,27 +4071,47 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="inlineStr"/>
-      <c r="G61" s="2" t="inlineStr"/>
-      <c r="H61" s="2" t="inlineStr"/>
-      <c r="I61" s="2" t="inlineStr"/>
-      <c r="J61" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>B02-G010</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -3931,27 +4131,47 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F62" s="2" t="inlineStr"/>
-      <c r="G62" s="2" t="inlineStr"/>
-      <c r="H62" s="2" t="inlineStr"/>
-      <c r="I62" s="2" t="inlineStr"/>
-      <c r="J62" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>B02-G011</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -3971,27 +4191,47 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr"/>
-      <c r="G63" s="2" t="inlineStr"/>
-      <c r="H63" s="2" t="inlineStr"/>
-      <c r="I63" s="2" t="inlineStr"/>
-      <c r="J63" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>B02-G012</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4011,27 +4251,47 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr"/>
-      <c r="G64" s="2" t="inlineStr"/>
-      <c r="H64" s="2" t="inlineStr"/>
-      <c r="I64" s="2" t="inlineStr"/>
-      <c r="J64" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>B02-G013</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4051,27 +4311,47 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F65" s="2" t="inlineStr"/>
-      <c r="G65" s="2" t="inlineStr"/>
-      <c r="H65" s="2" t="inlineStr"/>
-      <c r="I65" s="2" t="inlineStr"/>
-      <c r="J65" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>B02-G014</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4091,27 +4371,47 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="inlineStr"/>
-      <c r="G66" s="2" t="inlineStr"/>
-      <c r="H66" s="2" t="inlineStr"/>
-      <c r="I66" s="2" t="inlineStr"/>
-      <c r="J66" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>B02-G015; B02-G016</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4131,27 +4431,47 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="inlineStr"/>
-      <c r="G67" s="2" t="inlineStr"/>
-      <c r="H67" s="2" t="inlineStr"/>
-      <c r="I67" s="2" t="inlineStr"/>
-      <c r="J67" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>B02-G016; B02-G017</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4171,27 +4491,47 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr"/>
-      <c r="G68" s="2" t="inlineStr"/>
-      <c r="H68" s="2" t="inlineStr"/>
-      <c r="I68" s="2" t="inlineStr"/>
-      <c r="J68" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>B02-G018; B02-G019</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4211,27 +4551,47 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr"/>
-      <c r="G69" s="2" t="inlineStr"/>
-      <c r="H69" s="2" t="inlineStr"/>
-      <c r="I69" s="2" t="inlineStr"/>
-      <c r="J69" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>B02-G019</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4251,27 +4611,47 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr"/>
-      <c r="G70" s="2" t="inlineStr"/>
-      <c r="H70" s="2" t="inlineStr"/>
-      <c r="I70" s="2" t="inlineStr"/>
-      <c r="J70" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>B02-G019; B02-G020</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4291,27 +4671,47 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr"/>
-      <c r="G71" s="2" t="inlineStr"/>
-      <c r="H71" s="2" t="inlineStr"/>
-      <c r="I71" s="2" t="inlineStr"/>
-      <c r="J71" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>B02-G020</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4331,27 +4731,47 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr"/>
-      <c r="G72" s="2" t="inlineStr"/>
-      <c r="H72" s="2" t="inlineStr"/>
-      <c r="I72" s="2" t="inlineStr"/>
-      <c r="J72" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>B02-G021; B02-G022</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4371,27 +4791,47 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F73" s="2" t="inlineStr"/>
-      <c r="G73" s="2" t="inlineStr"/>
-      <c r="H73" s="2" t="inlineStr"/>
-      <c r="I73" s="2" t="inlineStr"/>
-      <c r="J73" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>B02-G023; B02-G024</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4411,27 +4851,47 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr"/>
-      <c r="G74" s="2" t="inlineStr"/>
-      <c r="H74" s="2" t="inlineStr"/>
-      <c r="I74" s="2" t="inlineStr"/>
-      <c r="J74" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>B02-G025</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4451,27 +4911,47 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr"/>
-      <c r="G75" s="2" t="inlineStr"/>
-      <c r="H75" s="2" t="inlineStr"/>
-      <c r="I75" s="2" t="inlineStr"/>
-      <c r="J75" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>B02-G026; B02-G027</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4491,27 +4971,47 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="inlineStr"/>
-      <c r="G76" s="2" t="inlineStr"/>
-      <c r="H76" s="2" t="inlineStr"/>
-      <c r="I76" s="2" t="inlineStr"/>
-      <c r="J76" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>B02-G028; B02-G029; B02-G030</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4531,27 +5031,47 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F77" s="2" t="inlineStr"/>
-      <c r="G77" s="2" t="inlineStr"/>
-      <c r="H77" s="2" t="inlineStr"/>
-      <c r="I77" s="2" t="inlineStr"/>
-      <c r="J77" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>B02-G031; B02-G032</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L77" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4571,27 +5091,47 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr"/>
-      <c r="G78" s="2" t="inlineStr"/>
-      <c r="H78" s="2" t="inlineStr"/>
-      <c r="I78" s="2" t="inlineStr"/>
-      <c r="J78" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>B02-G033; B02-G034</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4611,27 +5151,47 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F79" s="2" t="inlineStr"/>
-      <c r="G79" s="2" t="inlineStr"/>
-      <c r="H79" s="2" t="inlineStr"/>
-      <c r="I79" s="2" t="inlineStr"/>
-      <c r="J79" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>B02-G035; B02-G036</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4651,27 +5211,47 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr"/>
-      <c r="G80" s="2" t="inlineStr"/>
-      <c r="H80" s="2" t="inlineStr"/>
-      <c r="I80" s="2" t="inlineStr"/>
-      <c r="J80" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>B02-G037</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4691,27 +5271,47 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F81" s="2" t="inlineStr"/>
-      <c r="G81" s="2" t="inlineStr"/>
-      <c r="H81" s="2" t="inlineStr"/>
-      <c r="I81" s="2" t="inlineStr"/>
-      <c r="J81" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>B02-G038</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4731,27 +5331,47 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr"/>
-      <c r="G82" s="2" t="inlineStr"/>
-      <c r="H82" s="2" t="inlineStr"/>
-      <c r="I82" s="2" t="inlineStr"/>
-      <c r="J82" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>B02-G039</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4771,27 +5391,47 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F83" s="2" t="inlineStr"/>
-      <c r="G83" s="2" t="inlineStr"/>
-      <c r="H83" s="2" t="inlineStr"/>
-      <c r="I83" s="2" t="inlineStr"/>
-      <c r="J83" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>B02-G040</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K83" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4811,27 +5451,47 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr"/>
-      <c r="G84" s="2" t="inlineStr"/>
-      <c r="H84" s="2" t="inlineStr"/>
-      <c r="I84" s="2" t="inlineStr"/>
-      <c r="J84" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>B02-G041; B02-G042</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L84" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4851,27 +5511,47 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F85" s="2" t="inlineStr"/>
-      <c r="G85" s="2" t="inlineStr"/>
-      <c r="H85" s="2" t="inlineStr"/>
-      <c r="I85" s="2" t="inlineStr"/>
-      <c r="J85" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>B02-G042; B02-G043</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4891,27 +5571,47 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F86" s="2" t="inlineStr"/>
-      <c r="G86" s="2" t="inlineStr"/>
-      <c r="H86" s="2" t="inlineStr"/>
-      <c r="I86" s="2" t="inlineStr"/>
-      <c r="J86" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>B02-G044; B02-G045</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4931,27 +5631,47 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F87" s="2" t="inlineStr"/>
-      <c r="G87" s="2" t="inlineStr"/>
-      <c r="H87" s="2" t="inlineStr"/>
-      <c r="I87" s="2" t="inlineStr"/>
-      <c r="J87" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>B02-G046</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -4971,27 +5691,47 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F88" s="2" t="inlineStr"/>
-      <c r="G88" s="2" t="inlineStr"/>
-      <c r="H88" s="2" t="inlineStr"/>
-      <c r="I88" s="2" t="inlineStr"/>
-      <c r="J88" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>B02-G047; B02-G048</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L88" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -5011,27 +5751,47 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F89" s="2" t="inlineStr"/>
-      <c r="G89" s="2" t="inlineStr"/>
-      <c r="H89" s="2" t="inlineStr"/>
-      <c r="I89" s="2" t="inlineStr"/>
-      <c r="J89" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>B02-G049</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K89" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L89" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -5051,27 +5811,47 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F90" s="2" t="inlineStr"/>
-      <c r="G90" s="2" t="inlineStr"/>
-      <c r="H90" s="2" t="inlineStr"/>
-      <c r="I90" s="2" t="inlineStr"/>
-      <c r="J90" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>B02-G050</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L90" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -5091,27 +5871,47 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F91" s="2" t="inlineStr"/>
-      <c r="G91" s="2" t="inlineStr"/>
-      <c r="H91" s="2" t="inlineStr"/>
-      <c r="I91" s="2" t="inlineStr"/>
-      <c r="J91" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>B02-G051; B02-G052</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K91" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L91" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -5131,27 +5931,47 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F92" s="2" t="inlineStr"/>
-      <c r="G92" s="2" t="inlineStr"/>
-      <c r="H92" s="2" t="inlineStr"/>
-      <c r="I92" s="2" t="inlineStr"/>
-      <c r="J92" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>B02-G053; B02-G054</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -5171,27 +5991,47 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F93" s="2" t="inlineStr"/>
-      <c r="G93" s="2" t="inlineStr"/>
-      <c r="H93" s="2" t="inlineStr"/>
-      <c r="I93" s="2" t="inlineStr"/>
-      <c r="J93" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>B02-G054; B02-G055; B02-G056</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K93" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L93" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -5211,27 +6051,47 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F94" s="2" t="inlineStr"/>
-      <c r="G94" s="2" t="inlineStr"/>
-      <c r="H94" s="2" t="inlineStr"/>
-      <c r="I94" s="2" t="inlineStr"/>
-      <c r="J94" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>B02-G057</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -5251,27 +6111,47 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F95" s="2" t="inlineStr"/>
-      <c r="G95" s="2" t="inlineStr"/>
-      <c r="H95" s="2" t="inlineStr"/>
-      <c r="I95" s="2" t="inlineStr"/>
-      <c r="J95" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>B02-G058; B02-G059</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K95" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L95" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -5291,27 +6171,47 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F96" s="2" t="inlineStr"/>
-      <c r="G96" s="2" t="inlineStr"/>
-      <c r="H96" s="2" t="inlineStr"/>
-      <c r="I96" s="2" t="inlineStr"/>
-      <c r="J96" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>B02-G060</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K96" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -5331,27 +6231,47 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F97" s="2" t="inlineStr"/>
-      <c r="G97" s="2" t="inlineStr"/>
-      <c r="H97" s="2" t="inlineStr"/>
-      <c r="I97" s="2" t="inlineStr"/>
-      <c r="J97" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>B02-G061; B02-G062</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K97" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L97" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -5371,27 +6291,47 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F98" s="2" t="inlineStr"/>
-      <c r="G98" s="2" t="inlineStr"/>
-      <c r="H98" s="2" t="inlineStr"/>
-      <c r="I98" s="2" t="inlineStr"/>
-      <c r="J98" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>B02-G062; B02-G063</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K98" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L98" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -5411,27 +6351,47 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F99" s="2" t="inlineStr"/>
-      <c r="G99" s="2" t="inlineStr"/>
-      <c r="H99" s="2" t="inlineStr"/>
-      <c r="I99" s="2" t="inlineStr"/>
-      <c r="J99" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>B02-G064</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L99" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -5451,27 +6411,47 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F100" s="2" t="inlineStr"/>
-      <c r="G100" s="2" t="inlineStr"/>
-      <c r="H100" s="2" t="inlineStr"/>
-      <c r="I100" s="2" t="inlineStr"/>
-      <c r="J100" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>B02-G065</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K100" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L100" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>
@@ -5491,27 +6471,47 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F101" s="2" t="inlineStr"/>
-      <c r="G101" s="2" t="inlineStr"/>
-      <c r="H101" s="2" t="inlineStr"/>
-      <c r="I101" s="2" t="inlineStr"/>
-      <c r="J101" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>B02-G066; B02-G067</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K101" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L101" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared and OCR attempted only as an aid. Separate instruments on shared pages are listed separately.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Section 32 batch 03 checkpoint
Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
+++ b/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
@@ -6531,27 +6531,47 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F102" s="2" t="inlineStr"/>
-      <c r="G102" s="2" t="inlineStr"/>
-      <c r="H102" s="2" t="inlineStr"/>
-      <c r="I102" s="2" t="inlineStr"/>
-      <c r="J102" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>B02-G067; B03-G001; B03-G002</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K102" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L102" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -6571,27 +6591,47 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F103" s="2" t="inlineStr"/>
-      <c r="G103" s="2" t="inlineStr"/>
-      <c r="H103" s="2" t="inlineStr"/>
-      <c r="I103" s="2" t="inlineStr"/>
-      <c r="J103" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>B03-G003; B03-G004</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K103" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L103" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -6611,27 +6651,47 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F104" s="2" t="inlineStr"/>
-      <c r="G104" s="2" t="inlineStr"/>
-      <c r="H104" s="2" t="inlineStr"/>
-      <c r="I104" s="2" t="inlineStr"/>
-      <c r="J104" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>B03-G005</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K104" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L104" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -6651,27 +6711,47 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F105" s="2" t="inlineStr"/>
-      <c r="G105" s="2" t="inlineStr"/>
-      <c r="H105" s="2" t="inlineStr"/>
-      <c r="I105" s="2" t="inlineStr"/>
-      <c r="J105" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>B03-G006; B03-G007</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K105" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L105" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -6691,27 +6771,47 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F106" s="2" t="inlineStr"/>
-      <c r="G106" s="2" t="inlineStr"/>
-      <c r="H106" s="2" t="inlineStr"/>
-      <c r="I106" s="2" t="inlineStr"/>
-      <c r="J106" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>B03-G008; B03-G009</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K106" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L106" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -6731,27 +6831,47 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F107" s="2" t="inlineStr"/>
-      <c r="G107" s="2" t="inlineStr"/>
-      <c r="H107" s="2" t="inlineStr"/>
-      <c r="I107" s="2" t="inlineStr"/>
-      <c r="J107" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>B03-G010</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K107" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L107" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -6771,27 +6891,47 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F108" s="2" t="inlineStr"/>
-      <c r="G108" s="2" t="inlineStr"/>
-      <c r="H108" s="2" t="inlineStr"/>
-      <c r="I108" s="2" t="inlineStr"/>
-      <c r="J108" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>B03-G011</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K108" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L108" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -6811,27 +6951,47 @@
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F109" s="2" t="inlineStr"/>
-      <c r="G109" s="2" t="inlineStr"/>
-      <c r="H109" s="2" t="inlineStr"/>
-      <c r="I109" s="2" t="inlineStr"/>
-      <c r="J109" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>B03-G012; B03-G013</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K109" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L109" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -6851,27 +7011,47 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F110" s="2" t="inlineStr"/>
-      <c r="G110" s="2" t="inlineStr"/>
-      <c r="H110" s="2" t="inlineStr"/>
-      <c r="I110" s="2" t="inlineStr"/>
-      <c r="J110" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>B03-G014; B03-G015</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K110" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L110" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -6891,27 +7071,47 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F111" s="2" t="inlineStr"/>
-      <c r="G111" s="2" t="inlineStr"/>
-      <c r="H111" s="2" t="inlineStr"/>
-      <c r="I111" s="2" t="inlineStr"/>
-      <c r="J111" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>B03-G016; B03-G017</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K111" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L111" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -6931,27 +7131,47 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F112" s="2" t="inlineStr"/>
-      <c r="G112" s="2" t="inlineStr"/>
-      <c r="H112" s="2" t="inlineStr"/>
-      <c r="I112" s="2" t="inlineStr"/>
-      <c r="J112" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>B03-G018</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K112" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L112" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -6971,27 +7191,47 @@
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F113" s="2" t="inlineStr"/>
-      <c r="G113" s="2" t="inlineStr"/>
-      <c r="H113" s="2" t="inlineStr"/>
-      <c r="I113" s="2" t="inlineStr"/>
-      <c r="J113" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>B03-G019</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K113" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L113" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7011,27 +7251,47 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F114" s="2" t="inlineStr"/>
-      <c r="G114" s="2" t="inlineStr"/>
-      <c r="H114" s="2" t="inlineStr"/>
-      <c r="I114" s="2" t="inlineStr"/>
-      <c r="J114" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>B03-G020</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K114" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L114" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7051,27 +7311,47 @@
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F115" s="2" t="inlineStr"/>
-      <c r="G115" s="2" t="inlineStr"/>
-      <c r="H115" s="2" t="inlineStr"/>
-      <c r="I115" s="2" t="inlineStr"/>
-      <c r="J115" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>B03-G021; B03-G022</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I115" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J115" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K115" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L115" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7091,27 +7371,47 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F116" s="2" t="inlineStr"/>
-      <c r="G116" s="2" t="inlineStr"/>
-      <c r="H116" s="2" t="inlineStr"/>
-      <c r="I116" s="2" t="inlineStr"/>
-      <c r="J116" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>B03-G023</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J116" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K116" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L116" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7131,27 +7431,47 @@
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F117" s="2" t="inlineStr"/>
-      <c r="G117" s="2" t="inlineStr"/>
-      <c r="H117" s="2" t="inlineStr"/>
-      <c r="I117" s="2" t="inlineStr"/>
-      <c r="J117" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>B03-G024; B03-G025; B03-G026</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K117" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L117" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7171,27 +7491,47 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F118" s="2" t="inlineStr"/>
-      <c r="G118" s="2" t="inlineStr"/>
-      <c r="H118" s="2" t="inlineStr"/>
-      <c r="I118" s="2" t="inlineStr"/>
-      <c r="J118" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>B03-G026; B03-G027</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K118" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L118" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7211,27 +7551,47 @@
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F119" s="2" t="inlineStr"/>
-      <c r="G119" s="2" t="inlineStr"/>
-      <c r="H119" s="2" t="inlineStr"/>
-      <c r="I119" s="2" t="inlineStr"/>
-      <c r="J119" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>B03-G028</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J119" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K119" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L119" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7251,27 +7611,47 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F120" s="2" t="inlineStr"/>
-      <c r="G120" s="2" t="inlineStr"/>
-      <c r="H120" s="2" t="inlineStr"/>
-      <c r="I120" s="2" t="inlineStr"/>
-      <c r="J120" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>B03-G029; B03-G030</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K120" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L120" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7291,27 +7671,47 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F121" s="2" t="inlineStr"/>
-      <c r="G121" s="2" t="inlineStr"/>
-      <c r="H121" s="2" t="inlineStr"/>
-      <c r="I121" s="2" t="inlineStr"/>
-      <c r="J121" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>B03-G030; B03-G031</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J121" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K121" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L121" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7331,27 +7731,47 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F122" s="2" t="inlineStr"/>
-      <c r="G122" s="2" t="inlineStr"/>
-      <c r="H122" s="2" t="inlineStr"/>
-      <c r="I122" s="2" t="inlineStr"/>
-      <c r="J122" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>B03-G032; B03-G033</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J122" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K122" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L122" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7371,27 +7791,47 @@
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F123" s="2" t="inlineStr"/>
-      <c r="G123" s="2" t="inlineStr"/>
-      <c r="H123" s="2" t="inlineStr"/>
-      <c r="I123" s="2" t="inlineStr"/>
-      <c r="J123" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H123" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I123" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J123" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K123" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L123" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7411,27 +7851,47 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F124" s="2" t="inlineStr"/>
-      <c r="G124" s="2" t="inlineStr"/>
-      <c r="H124" s="2" t="inlineStr"/>
-      <c r="I124" s="2" t="inlineStr"/>
-      <c r="J124" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J124" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K124" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L124" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7451,27 +7911,47 @@
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F125" s="2" t="inlineStr"/>
-      <c r="G125" s="2" t="inlineStr"/>
-      <c r="H125" s="2" t="inlineStr"/>
-      <c r="I125" s="2" t="inlineStr"/>
-      <c r="J125" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J125" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K125" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L125" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7491,27 +7971,47 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F126" s="2" t="inlineStr"/>
-      <c r="G126" s="2" t="inlineStr"/>
-      <c r="H126" s="2" t="inlineStr"/>
-      <c r="I126" s="2" t="inlineStr"/>
-      <c r="J126" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J126" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K126" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L126" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7531,27 +8031,47 @@
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F127" s="2" t="inlineStr"/>
-      <c r="G127" s="2" t="inlineStr"/>
-      <c r="H127" s="2" t="inlineStr"/>
-      <c r="I127" s="2" t="inlineStr"/>
-      <c r="J127" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I127" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J127" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K127" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L127" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7571,27 +8091,47 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F128" s="2" t="inlineStr"/>
-      <c r="G128" s="2" t="inlineStr"/>
-      <c r="H128" s="2" t="inlineStr"/>
-      <c r="I128" s="2" t="inlineStr"/>
-      <c r="J128" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J128" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K128" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L128" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7611,27 +8151,47 @@
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F129" s="2" t="inlineStr"/>
-      <c r="G129" s="2" t="inlineStr"/>
-      <c r="H129" s="2" t="inlineStr"/>
-      <c r="I129" s="2" t="inlineStr"/>
-      <c r="J129" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J129" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K129" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L129" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7651,27 +8211,47 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F130" s="2" t="inlineStr"/>
-      <c r="G130" s="2" t="inlineStr"/>
-      <c r="H130" s="2" t="inlineStr"/>
-      <c r="I130" s="2" t="inlineStr"/>
-      <c r="J130" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J130" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K130" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L130" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7691,27 +8271,47 @@
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F131" s="2" t="inlineStr"/>
-      <c r="G131" s="2" t="inlineStr"/>
-      <c r="H131" s="2" t="inlineStr"/>
-      <c r="I131" s="2" t="inlineStr"/>
-      <c r="J131" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J131" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K131" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L131" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7731,27 +8331,47 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F132" s="2" t="inlineStr"/>
-      <c r="G132" s="2" t="inlineStr"/>
-      <c r="H132" s="2" t="inlineStr"/>
-      <c r="I132" s="2" t="inlineStr"/>
-      <c r="J132" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J132" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K132" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L132" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7771,27 +8391,47 @@
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F133" s="2" t="inlineStr"/>
-      <c r="G133" s="2" t="inlineStr"/>
-      <c r="H133" s="2" t="inlineStr"/>
-      <c r="I133" s="2" t="inlineStr"/>
-      <c r="J133" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H133" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J133" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K133" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L133" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7811,27 +8451,47 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F134" s="2" t="inlineStr"/>
-      <c r="G134" s="2" t="inlineStr"/>
-      <c r="H134" s="2" t="inlineStr"/>
-      <c r="I134" s="2" t="inlineStr"/>
-      <c r="J134" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J134" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K134" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L134" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7851,27 +8511,47 @@
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F135" s="2" t="inlineStr"/>
-      <c r="G135" s="2" t="inlineStr"/>
-      <c r="H135" s="2" t="inlineStr"/>
-      <c r="I135" s="2" t="inlineStr"/>
-      <c r="J135" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H135" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J135" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K135" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L135" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7891,27 +8571,47 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F136" s="2" t="inlineStr"/>
-      <c r="G136" s="2" t="inlineStr"/>
-      <c r="H136" s="2" t="inlineStr"/>
-      <c r="I136" s="2" t="inlineStr"/>
-      <c r="J136" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K136" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L136" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7931,27 +8631,47 @@
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F137" s="2" t="inlineStr"/>
-      <c r="G137" s="2" t="inlineStr"/>
-      <c r="H137" s="2" t="inlineStr"/>
-      <c r="I137" s="2" t="inlineStr"/>
-      <c r="J137" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K137" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L137" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -7971,27 +8691,47 @@
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F138" s="2" t="inlineStr"/>
-      <c r="G138" s="2" t="inlineStr"/>
-      <c r="H138" s="2" t="inlineStr"/>
-      <c r="I138" s="2" t="inlineStr"/>
-      <c r="J138" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J138" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K138" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L138" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -8011,27 +8751,47 @@
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F139" s="2" t="inlineStr"/>
-      <c r="G139" s="2" t="inlineStr"/>
-      <c r="H139" s="2" t="inlineStr"/>
-      <c r="I139" s="2" t="inlineStr"/>
-      <c r="J139" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K139" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L139" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -8051,27 +8811,47 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F140" s="2" t="inlineStr"/>
-      <c r="G140" s="2" t="inlineStr"/>
-      <c r="H140" s="2" t="inlineStr"/>
-      <c r="I140" s="2" t="inlineStr"/>
-      <c r="J140" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K140" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L140" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -8091,27 +8871,47 @@
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F141" s="2" t="inlineStr"/>
-      <c r="G141" s="2" t="inlineStr"/>
-      <c r="H141" s="2" t="inlineStr"/>
-      <c r="I141" s="2" t="inlineStr"/>
-      <c r="J141" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K141" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L141" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -8131,27 +8931,47 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F142" s="2" t="inlineStr"/>
-      <c r="G142" s="2" t="inlineStr"/>
-      <c r="H142" s="2" t="inlineStr"/>
-      <c r="I142" s="2" t="inlineStr"/>
-      <c r="J142" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K142" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L142" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -8171,27 +8991,47 @@
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F143" s="2" t="inlineStr"/>
-      <c r="G143" s="2" t="inlineStr"/>
-      <c r="H143" s="2" t="inlineStr"/>
-      <c r="I143" s="2" t="inlineStr"/>
-      <c r="J143" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J143" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -8211,27 +9051,47 @@
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F144" s="2" t="inlineStr"/>
-      <c r="G144" s="2" t="inlineStr"/>
-      <c r="H144" s="2" t="inlineStr"/>
-      <c r="I144" s="2" t="inlineStr"/>
-      <c r="J144" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>B03-G034; B03-G035</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -8251,27 +9111,47 @@
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F145" s="2" t="inlineStr"/>
-      <c r="G145" s="2" t="inlineStr"/>
-      <c r="H145" s="2" t="inlineStr"/>
-      <c r="I145" s="2" t="inlineStr"/>
-      <c r="J145" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>B03-G036</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K145" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L145" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -8291,27 +9171,47 @@
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F146" s="2" t="inlineStr"/>
-      <c r="G146" s="2" t="inlineStr"/>
-      <c r="H146" s="2" t="inlineStr"/>
-      <c r="I146" s="2" t="inlineStr"/>
-      <c r="J146" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>B03-G037</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J146" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K146" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L146" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -8331,27 +9231,47 @@
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F147" s="2" t="inlineStr"/>
-      <c r="G147" s="2" t="inlineStr"/>
-      <c r="H147" s="2" t="inlineStr"/>
-      <c r="I147" s="2" t="inlineStr"/>
-      <c r="J147" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>B03-G038</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J147" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K147" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L147" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -8371,27 +9291,47 @@
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F148" s="2" t="inlineStr"/>
-      <c r="G148" s="2" t="inlineStr"/>
-      <c r="H148" s="2" t="inlineStr"/>
-      <c r="I148" s="2" t="inlineStr"/>
-      <c r="J148" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>B03-G039</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J148" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K148" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L148" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -8411,27 +9351,47 @@
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F149" s="2" t="inlineStr"/>
-      <c r="G149" s="2" t="inlineStr"/>
-      <c r="H149" s="2" t="inlineStr"/>
-      <c r="I149" s="2" t="inlineStr"/>
-      <c r="J149" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>B03-G040</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J149" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K149" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L149" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -8451,27 +9411,47 @@
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F150" s="2" t="inlineStr"/>
-      <c r="G150" s="2" t="inlineStr"/>
-      <c r="H150" s="2" t="inlineStr"/>
-      <c r="I150" s="2" t="inlineStr"/>
-      <c r="J150" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I150" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J150" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K150" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L150" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -8491,27 +9471,47 @@
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F151" s="2" t="inlineStr"/>
-      <c r="G151" s="2" t="inlineStr"/>
-      <c r="H151" s="2" t="inlineStr"/>
-      <c r="I151" s="2" t="inlineStr"/>
-      <c r="J151" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J151" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K151" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L151" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Section 32 batch 04 checkpoint
Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
+++ b/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
@@ -9531,27 +9531,47 @@
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F152" s="2" t="inlineStr"/>
-      <c r="G152" s="2" t="inlineStr"/>
-      <c r="H152" s="2" t="inlineStr"/>
-      <c r="I152" s="2" t="inlineStr"/>
-      <c r="J152" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J152" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K152" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L152" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -9571,27 +9591,47 @@
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F153" s="2" t="inlineStr"/>
-      <c r="G153" s="2" t="inlineStr"/>
-      <c r="H153" s="2" t="inlineStr"/>
-      <c r="I153" s="2" t="inlineStr"/>
-      <c r="J153" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I153" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J153" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K153" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L153" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -9611,27 +9651,47 @@
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F154" s="2" t="inlineStr"/>
-      <c r="G154" s="2" t="inlineStr"/>
-      <c r="H154" s="2" t="inlineStr"/>
-      <c r="I154" s="2" t="inlineStr"/>
-      <c r="J154" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J154" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K154" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L154" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -9651,27 +9711,47 @@
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F155" s="2" t="inlineStr"/>
-      <c r="G155" s="2" t="inlineStr"/>
-      <c r="H155" s="2" t="inlineStr"/>
-      <c r="I155" s="2" t="inlineStr"/>
-      <c r="J155" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I155" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J155" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K155" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L155" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -9691,27 +9771,47 @@
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F156" s="2" t="inlineStr"/>
-      <c r="G156" s="2" t="inlineStr"/>
-      <c r="H156" s="2" t="inlineStr"/>
-      <c r="I156" s="2" t="inlineStr"/>
-      <c r="J156" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J156" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K156" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L156" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -9731,27 +9831,47 @@
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F157" s="2" t="inlineStr"/>
-      <c r="G157" s="2" t="inlineStr"/>
-      <c r="H157" s="2" t="inlineStr"/>
-      <c r="I157" s="2" t="inlineStr"/>
-      <c r="J157" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G157" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H157" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I157" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J157" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K157" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L157" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -9771,27 +9891,47 @@
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F158" s="2" t="inlineStr"/>
-      <c r="G158" s="2" t="inlineStr"/>
-      <c r="H158" s="2" t="inlineStr"/>
-      <c r="I158" s="2" t="inlineStr"/>
-      <c r="J158" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I158" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J158" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K158" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L158" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -9811,27 +9951,47 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F159" s="2" t="inlineStr"/>
-      <c r="G159" s="2" t="inlineStr"/>
-      <c r="H159" s="2" t="inlineStr"/>
-      <c r="I159" s="2" t="inlineStr"/>
-      <c r="J159" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G159" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H159" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I159" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J159" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K159" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L159" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -9851,27 +10011,47 @@
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F160" s="2" t="inlineStr"/>
-      <c r="G160" s="2" t="inlineStr"/>
-      <c r="H160" s="2" t="inlineStr"/>
-      <c r="I160" s="2" t="inlineStr"/>
-      <c r="J160" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I160" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J160" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K160" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L160" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -9891,27 +10071,47 @@
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F161" s="2" t="inlineStr"/>
-      <c r="G161" s="2" t="inlineStr"/>
-      <c r="H161" s="2" t="inlineStr"/>
-      <c r="I161" s="2" t="inlineStr"/>
-      <c r="J161" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G161" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I161" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J161" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K161" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L161" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -9931,27 +10131,47 @@
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F162" s="2" t="inlineStr"/>
-      <c r="G162" s="2" t="inlineStr"/>
-      <c r="H162" s="2" t="inlineStr"/>
-      <c r="I162" s="2" t="inlineStr"/>
-      <c r="J162" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I162" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J162" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K162" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L162" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -9971,27 +10191,47 @@
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F163" s="2" t="inlineStr"/>
-      <c r="G163" s="2" t="inlineStr"/>
-      <c r="H163" s="2" t="inlineStr"/>
-      <c r="I163" s="2" t="inlineStr"/>
-      <c r="J163" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I163" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J163" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K163" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L163" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10011,27 +10251,47 @@
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F164" s="2" t="inlineStr"/>
-      <c r="G164" s="2" t="inlineStr"/>
-      <c r="H164" s="2" t="inlineStr"/>
-      <c r="I164" s="2" t="inlineStr"/>
-      <c r="J164" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H164" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I164" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J164" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K164" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L164" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10051,27 +10311,47 @@
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F165" s="2" t="inlineStr"/>
-      <c r="G165" s="2" t="inlineStr"/>
-      <c r="H165" s="2" t="inlineStr"/>
-      <c r="I165" s="2" t="inlineStr"/>
-      <c r="J165" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I165" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J165" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K165" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L165" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10091,27 +10371,47 @@
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F166" s="2" t="inlineStr"/>
-      <c r="G166" s="2" t="inlineStr"/>
-      <c r="H166" s="2" t="inlineStr"/>
-      <c r="I166" s="2" t="inlineStr"/>
-      <c r="J166" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I166" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J166" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K166" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L166" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10131,27 +10431,47 @@
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E167" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F167" s="2" t="inlineStr"/>
-      <c r="G167" s="2" t="inlineStr"/>
-      <c r="H167" s="2" t="inlineStr"/>
-      <c r="I167" s="2" t="inlineStr"/>
-      <c r="J167" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H167" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I167" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J167" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K167" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L167" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10171,27 +10491,47 @@
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F168" s="2" t="inlineStr"/>
-      <c r="G168" s="2" t="inlineStr"/>
-      <c r="H168" s="2" t="inlineStr"/>
-      <c r="I168" s="2" t="inlineStr"/>
-      <c r="J168" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I168" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J168" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K168" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L168" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10211,27 +10551,47 @@
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F169" s="2" t="inlineStr"/>
-      <c r="G169" s="2" t="inlineStr"/>
-      <c r="H169" s="2" t="inlineStr"/>
-      <c r="I169" s="2" t="inlineStr"/>
-      <c r="J169" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041</t>
+        </is>
+      </c>
+      <c r="H169" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I169" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J169" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K169" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L169" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10251,27 +10611,47 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F170" s="2" t="inlineStr"/>
-      <c r="G170" s="2" t="inlineStr"/>
-      <c r="H170" s="2" t="inlineStr"/>
-      <c r="I170" s="2" t="inlineStr"/>
-      <c r="J170" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>B03-G041; B04-G001</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>continuation_and_first_page</t>
+        </is>
+      </c>
+      <c r="I170" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J170" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K170" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L170" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10291,27 +10671,47 @@
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E171" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F171" s="2" t="inlineStr"/>
-      <c r="G171" s="2" t="inlineStr"/>
-      <c r="H171" s="2" t="inlineStr"/>
-      <c r="I171" s="2" t="inlineStr"/>
-      <c r="J171" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>B04-G002; B04-G003</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="inlineStr">
+        <is>
+          <t>continuation_and_first_page</t>
+        </is>
+      </c>
+      <c r="I171" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J171" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K171" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L171" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10331,27 +10731,47 @@
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F172" s="2" t="inlineStr"/>
-      <c r="G172" s="2" t="inlineStr"/>
-      <c r="H172" s="2" t="inlineStr"/>
-      <c r="I172" s="2" t="inlineStr"/>
-      <c r="J172" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I172" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J172" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K172" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L172" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10371,27 +10791,47 @@
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F173" s="2" t="inlineStr"/>
-      <c r="G173" s="2" t="inlineStr"/>
-      <c r="H173" s="2" t="inlineStr"/>
-      <c r="I173" s="2" t="inlineStr"/>
-      <c r="J173" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I173" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J173" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K173" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L173" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10411,27 +10851,47 @@
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F174" s="2" t="inlineStr"/>
-      <c r="G174" s="2" t="inlineStr"/>
-      <c r="H174" s="2" t="inlineStr"/>
-      <c r="I174" s="2" t="inlineStr"/>
-      <c r="J174" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I174" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J174" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K174" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L174" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10451,27 +10911,47 @@
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E175" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F175" s="2" t="inlineStr"/>
-      <c r="G175" s="2" t="inlineStr"/>
-      <c r="H175" s="2" t="inlineStr"/>
-      <c r="I175" s="2" t="inlineStr"/>
-      <c r="J175" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I175" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J175" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K175" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L175" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10491,27 +10971,47 @@
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F176" s="2" t="inlineStr"/>
-      <c r="G176" s="2" t="inlineStr"/>
-      <c r="H176" s="2" t="inlineStr"/>
-      <c r="I176" s="2" t="inlineStr"/>
-      <c r="J176" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J176" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K176" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L176" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10531,27 +11031,47 @@
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F177" s="2" t="inlineStr"/>
-      <c r="G177" s="2" t="inlineStr"/>
-      <c r="H177" s="2" t="inlineStr"/>
-      <c r="I177" s="2" t="inlineStr"/>
-      <c r="J177" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I177" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J177" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K177" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L177" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10571,27 +11091,47 @@
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F178" s="2" t="inlineStr"/>
-      <c r="G178" s="2" t="inlineStr"/>
-      <c r="H178" s="2" t="inlineStr"/>
-      <c r="I178" s="2" t="inlineStr"/>
-      <c r="J178" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H178" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I178" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J178" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K178" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L178" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10611,27 +11151,47 @@
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E179" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F179" s="2" t="inlineStr"/>
-      <c r="G179" s="2" t="inlineStr"/>
-      <c r="H179" s="2" t="inlineStr"/>
-      <c r="I179" s="2" t="inlineStr"/>
-      <c r="J179" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I179" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K179" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L179" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10651,27 +11211,47 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F180" s="2" t="inlineStr"/>
-      <c r="G180" s="2" t="inlineStr"/>
-      <c r="H180" s="2" t="inlineStr"/>
-      <c r="I180" s="2" t="inlineStr"/>
-      <c r="J180" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K180" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L180" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10691,27 +11271,47 @@
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F181" s="2" t="inlineStr"/>
-      <c r="G181" s="2" t="inlineStr"/>
-      <c r="H181" s="2" t="inlineStr"/>
-      <c r="I181" s="2" t="inlineStr"/>
-      <c r="J181" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I181" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J181" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K181" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L181" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10731,27 +11331,47 @@
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F182" s="2" t="inlineStr"/>
-      <c r="G182" s="2" t="inlineStr"/>
-      <c r="H182" s="2" t="inlineStr"/>
-      <c r="I182" s="2" t="inlineStr"/>
-      <c r="J182" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K182" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L182" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10771,27 +11391,47 @@
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F183" s="2" t="inlineStr"/>
-      <c r="G183" s="2" t="inlineStr"/>
-      <c r="H183" s="2" t="inlineStr"/>
-      <c r="I183" s="2" t="inlineStr"/>
-      <c r="J183" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I183" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J183" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K183" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L183" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10811,27 +11451,47 @@
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F184" s="2" t="inlineStr"/>
-      <c r="G184" s="2" t="inlineStr"/>
-      <c r="H184" s="2" t="inlineStr"/>
-      <c r="I184" s="2" t="inlineStr"/>
-      <c r="J184" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I184" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K184" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L184" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10851,27 +11511,47 @@
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E185" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F185" s="2" t="inlineStr"/>
-      <c r="G185" s="2" t="inlineStr"/>
-      <c r="H185" s="2" t="inlineStr"/>
-      <c r="I185" s="2" t="inlineStr"/>
-      <c r="J185" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I185" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K185" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L185" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10891,27 +11571,47 @@
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E186" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F186" s="2" t="inlineStr"/>
-      <c r="G186" s="2" t="inlineStr"/>
-      <c r="H186" s="2" t="inlineStr"/>
-      <c r="I186" s="2" t="inlineStr"/>
-      <c r="J186" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I186" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K186" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L186" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10931,27 +11631,47 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E187" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F187" s="2" t="inlineStr"/>
-      <c r="G187" s="2" t="inlineStr"/>
-      <c r="H187" s="2" t="inlineStr"/>
-      <c r="I187" s="2" t="inlineStr"/>
-      <c r="J187" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I187" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K187" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L187" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -10971,27 +11691,47 @@
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F188" s="2" t="inlineStr"/>
-      <c r="G188" s="2" t="inlineStr"/>
-      <c r="H188" s="2" t="inlineStr"/>
-      <c r="I188" s="2" t="inlineStr"/>
-      <c r="J188" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I188" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K188" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L188" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -11011,27 +11751,47 @@
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E189" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F189" s="2" t="inlineStr"/>
-      <c r="G189" s="2" t="inlineStr"/>
-      <c r="H189" s="2" t="inlineStr"/>
-      <c r="I189" s="2" t="inlineStr"/>
-      <c r="J189" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G189" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I189" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J189" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K189" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L189" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -11051,27 +11811,47 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F190" s="2" t="inlineStr"/>
-      <c r="G190" s="2" t="inlineStr"/>
-      <c r="H190" s="2" t="inlineStr"/>
-      <c r="I190" s="2" t="inlineStr"/>
-      <c r="J190" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K190" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L190" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -11091,27 +11871,47 @@
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E191" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F191" s="2" t="inlineStr"/>
-      <c r="G191" s="2" t="inlineStr"/>
-      <c r="H191" s="2" t="inlineStr"/>
-      <c r="I191" s="2" t="inlineStr"/>
-      <c r="J191" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I191" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J191" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K191" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L191" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -11131,27 +11931,47 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E192" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F192" s="2" t="inlineStr"/>
-      <c r="G192" s="2" t="inlineStr"/>
-      <c r="H192" s="2" t="inlineStr"/>
-      <c r="I192" s="2" t="inlineStr"/>
-      <c r="J192" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I192" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J192" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K192" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L192" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -11171,27 +11991,47 @@
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E193" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F193" s="2" t="inlineStr"/>
-      <c r="G193" s="2" t="inlineStr"/>
-      <c r="H193" s="2" t="inlineStr"/>
-      <c r="I193" s="2" t="inlineStr"/>
-      <c r="J193" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F193" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G193" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I193" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J193" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -11211,27 +12051,47 @@
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F194" s="2" t="inlineStr"/>
-      <c r="G194" s="2" t="inlineStr"/>
-      <c r="H194" s="2" t="inlineStr"/>
-      <c r="I194" s="2" t="inlineStr"/>
-      <c r="J194" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G194" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I194" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J194" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K194" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L194" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -11251,27 +12111,47 @@
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F195" s="2" t="inlineStr"/>
-      <c r="G195" s="2" t="inlineStr"/>
-      <c r="H195" s="2" t="inlineStr"/>
-      <c r="I195" s="2" t="inlineStr"/>
-      <c r="J195" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F195" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G195" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I195" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J195" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -11291,27 +12171,47 @@
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F196" s="2" t="inlineStr"/>
-      <c r="G196" s="2" t="inlineStr"/>
-      <c r="H196" s="2" t="inlineStr"/>
-      <c r="I196" s="2" t="inlineStr"/>
-      <c r="J196" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H196" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I196" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J196" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K196" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L196" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -11331,27 +12231,47 @@
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E197" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F197" s="2" t="inlineStr"/>
-      <c r="G197" s="2" t="inlineStr"/>
-      <c r="H197" s="2" t="inlineStr"/>
-      <c r="I197" s="2" t="inlineStr"/>
-      <c r="J197" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F197" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G197" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H197" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I197" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J197" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K197" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L197" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -11371,27 +12291,47 @@
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F198" s="2" t="inlineStr"/>
-      <c r="G198" s="2" t="inlineStr"/>
-      <c r="H198" s="2" t="inlineStr"/>
-      <c r="I198" s="2" t="inlineStr"/>
-      <c r="J198" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I198" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J198" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K198" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L198" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -11411,27 +12351,47 @@
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F199" s="2" t="inlineStr"/>
-      <c r="G199" s="2" t="inlineStr"/>
-      <c r="H199" s="2" t="inlineStr"/>
-      <c r="I199" s="2" t="inlineStr"/>
-      <c r="J199" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I199" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J199" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K199" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L199" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -11451,27 +12411,47 @@
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F200" s="2" t="inlineStr"/>
-      <c r="G200" s="2" t="inlineStr"/>
-      <c r="H200" s="2" t="inlineStr"/>
-      <c r="I200" s="2" t="inlineStr"/>
-      <c r="J200" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I200" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J200" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K200" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L200" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>
@@ -11491,27 +12471,47 @@
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E201" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F201" s="2" t="inlineStr"/>
-      <c r="G201" s="2" t="inlineStr"/>
-      <c r="H201" s="2" t="inlineStr"/>
-      <c r="I201" s="2" t="inlineStr"/>
-      <c r="J201" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G201" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I201" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J201" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K201" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L201" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; adjacent pages compared. OCR and enhanced zoom/crops were used only as aids. Stamps, signatures, marginal notes, and schedule entries were checked; separate instruments sharing a page are listed separately.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Section 32 batch 05 checkpoint
Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
+++ b/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
@@ -12531,27 +12531,47 @@
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F202" s="2" t="inlineStr"/>
-      <c r="G202" s="2" t="inlineStr"/>
-      <c r="H202" s="2" t="inlineStr"/>
-      <c r="I202" s="2" t="inlineStr"/>
-      <c r="J202" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I202" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K202" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L202" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -12571,27 +12591,47 @@
       </c>
       <c r="D203" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F203" s="2" t="inlineStr"/>
-      <c r="G203" s="2" t="inlineStr"/>
-      <c r="H203" s="2" t="inlineStr"/>
-      <c r="I203" s="2" t="inlineStr"/>
-      <c r="J203" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I203" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J203" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K203" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L203" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -12611,27 +12651,47 @@
       </c>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E204" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F204" s="2" t="inlineStr"/>
-      <c r="G204" s="2" t="inlineStr"/>
-      <c r="H204" s="2" t="inlineStr"/>
-      <c r="I204" s="2" t="inlineStr"/>
-      <c r="J204" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I204" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J204" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K204" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L204" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -12651,27 +12711,47 @@
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E205" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F205" s="2" t="inlineStr"/>
-      <c r="G205" s="2" t="inlineStr"/>
-      <c r="H205" s="2" t="inlineStr"/>
-      <c r="I205" s="2" t="inlineStr"/>
-      <c r="J205" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H205" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I205" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J205" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K205" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L205" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -12691,27 +12771,47 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E206" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F206" s="2" t="inlineStr"/>
-      <c r="G206" s="2" t="inlineStr"/>
-      <c r="H206" s="2" t="inlineStr"/>
-      <c r="I206" s="2" t="inlineStr"/>
-      <c r="J206" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>poor/faint</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H206" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I206" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J206" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K206" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L206" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -12731,27 +12831,47 @@
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E207" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F207" s="2" t="inlineStr"/>
-      <c r="G207" s="2" t="inlineStr"/>
-      <c r="H207" s="2" t="inlineStr"/>
-      <c r="I207" s="2" t="inlineStr"/>
-      <c r="J207" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F207" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G207" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H207" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I207" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J207" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L207" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -12771,27 +12891,47 @@
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E208" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F208" s="2" t="inlineStr"/>
-      <c r="G208" s="2" t="inlineStr"/>
-      <c r="H208" s="2" t="inlineStr"/>
-      <c r="I208" s="2" t="inlineStr"/>
-      <c r="J208" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I208" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J208" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K208" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L208" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -12811,27 +12951,47 @@
       </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E209" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F209" s="2" t="inlineStr"/>
-      <c r="G209" s="2" t="inlineStr"/>
-      <c r="H209" s="2" t="inlineStr"/>
-      <c r="I209" s="2" t="inlineStr"/>
-      <c r="J209" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F209" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G209" s="2" t="inlineStr">
+        <is>
+          <t>B04-G003</t>
+        </is>
+      </c>
+      <c r="H209" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I209" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J209" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K209" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L209" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -12851,27 +13011,47 @@
       </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E210" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F210" s="2" t="inlineStr"/>
-      <c r="G210" s="2" t="inlineStr"/>
-      <c r="H210" s="2" t="inlineStr"/>
-      <c r="I210" s="2" t="inlineStr"/>
-      <c r="J210" s="2" t="inlineStr"/>
+          <t>new_instrument_page</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t>B05-G001</t>
+        </is>
+      </c>
+      <c r="H210" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I210" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J210" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K210" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L210" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -12891,27 +13071,47 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E211" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F211" s="2" t="inlineStr"/>
-      <c r="G211" s="2" t="inlineStr"/>
-      <c r="H211" s="2" t="inlineStr"/>
-      <c r="I211" s="2" t="inlineStr"/>
-      <c r="J211" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t>B05-G002; B05-G003</t>
+        </is>
+      </c>
+      <c r="H211" s="2" t="inlineStr">
+        <is>
+          <t>continuation_and_first_page</t>
+        </is>
+      </c>
+      <c r="I211" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J211" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K211" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L211" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -12931,27 +13131,47 @@
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E212" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F212" s="2" t="inlineStr"/>
-      <c r="G212" s="2" t="inlineStr"/>
-      <c r="H212" s="2" t="inlineStr"/>
-      <c r="I212" s="2" t="inlineStr"/>
-      <c r="J212" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F212" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G212" s="2" t="inlineStr">
+        <is>
+          <t>B05-G003</t>
+        </is>
+      </c>
+      <c r="H212" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I212" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J212" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K212" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L212" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -12971,27 +13191,47 @@
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E213" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F213" s="2" t="inlineStr"/>
-      <c r="G213" s="2" t="inlineStr"/>
-      <c r="H213" s="2" t="inlineStr"/>
-      <c r="I213" s="2" t="inlineStr"/>
-      <c r="J213" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
+          <t>B05-G003; B05-G004</t>
+        </is>
+      </c>
+      <c r="H213" s="2" t="inlineStr">
+        <is>
+          <t>continuation_and_first_page</t>
+        </is>
+      </c>
+      <c r="I213" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J213" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K213" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L213" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13011,27 +13251,47 @@
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E214" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F214" s="2" t="inlineStr"/>
-      <c r="G214" s="2" t="inlineStr"/>
-      <c r="H214" s="2" t="inlineStr"/>
-      <c r="I214" s="2" t="inlineStr"/>
-      <c r="J214" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G214" s="2" t="inlineStr">
+        <is>
+          <t>B05-G004</t>
+        </is>
+      </c>
+      <c r="H214" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I214" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J214" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K214" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L214" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13051,27 +13311,47 @@
       </c>
       <c r="D215" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E215" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F215" s="2" t="inlineStr"/>
-      <c r="G215" s="2" t="inlineStr"/>
-      <c r="H215" s="2" t="inlineStr"/>
-      <c r="I215" s="2" t="inlineStr"/>
-      <c r="J215" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F215" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G215" s="2" t="inlineStr">
+        <is>
+          <t>B05-G004; B05-G005</t>
+        </is>
+      </c>
+      <c r="H215" s="2" t="inlineStr">
+        <is>
+          <t>continuation_and_first_page</t>
+        </is>
+      </c>
+      <c r="I215" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J215" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K215" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L215" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13091,27 +13371,47 @@
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E216" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F216" s="2" t="inlineStr"/>
-      <c r="G216" s="2" t="inlineStr"/>
-      <c r="H216" s="2" t="inlineStr"/>
-      <c r="I216" s="2" t="inlineStr"/>
-      <c r="J216" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G216" s="2" t="inlineStr">
+        <is>
+          <t>B05-G006; B05-G007</t>
+        </is>
+      </c>
+      <c r="H216" s="2" t="inlineStr">
+        <is>
+          <t>multiple_first_pages</t>
+        </is>
+      </c>
+      <c r="I216" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J216" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K216" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L216" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13131,27 +13431,47 @@
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E217" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F217" s="2" t="inlineStr"/>
-      <c r="G217" s="2" t="inlineStr"/>
-      <c r="H217" s="2" t="inlineStr"/>
-      <c r="I217" s="2" t="inlineStr"/>
-      <c r="J217" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F217" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G217" s="2" t="inlineStr">
+        <is>
+          <t>B05-G007; B05-G008</t>
+        </is>
+      </c>
+      <c r="H217" s="2" t="inlineStr">
+        <is>
+          <t>continuation_and_first_page</t>
+        </is>
+      </c>
+      <c r="I217" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J217" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K217" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L217" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13171,27 +13491,47 @@
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F218" s="2" t="inlineStr"/>
-      <c r="G218" s="2" t="inlineStr"/>
-      <c r="H218" s="2" t="inlineStr"/>
-      <c r="I218" s="2" t="inlineStr"/>
-      <c r="J218" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F218" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G218" s="2" t="inlineStr">
+        <is>
+          <t>B05-G009; B05-G010</t>
+        </is>
+      </c>
+      <c r="H218" s="2" t="inlineStr">
+        <is>
+          <t>multiple_first_pages</t>
+        </is>
+      </c>
+      <c r="I218" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J218" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K218" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L218" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13211,27 +13551,47 @@
       </c>
       <c r="D219" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E219" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F219" s="2" t="inlineStr"/>
-      <c r="G219" s="2" t="inlineStr"/>
-      <c r="H219" s="2" t="inlineStr"/>
-      <c r="I219" s="2" t="inlineStr"/>
-      <c r="J219" s="2" t="inlineStr"/>
+          <t>new_instrument_page</t>
+        </is>
+      </c>
+      <c r="F219" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G219" s="2" t="inlineStr">
+        <is>
+          <t>B05-G011</t>
+        </is>
+      </c>
+      <c r="H219" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I219" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J219" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K219" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L219" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13251,27 +13611,47 @@
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F220" s="2" t="inlineStr"/>
-      <c r="G220" s="2" t="inlineStr"/>
-      <c r="H220" s="2" t="inlineStr"/>
-      <c r="I220" s="2" t="inlineStr"/>
-      <c r="J220" s="2" t="inlineStr"/>
+          <t>new_instrument_page</t>
+        </is>
+      </c>
+      <c r="F220" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G220" s="2" t="inlineStr">
+        <is>
+          <t>B05-G012</t>
+        </is>
+      </c>
+      <c r="H220" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I220" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J220" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K220" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L220" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13291,27 +13671,47 @@
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E221" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F221" s="2" t="inlineStr"/>
-      <c r="G221" s="2" t="inlineStr"/>
-      <c r="H221" s="2" t="inlineStr"/>
-      <c r="I221" s="2" t="inlineStr"/>
-      <c r="J221" s="2" t="inlineStr"/>
+          <t>new_instrument_page</t>
+        </is>
+      </c>
+      <c r="F221" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G221" s="2" t="inlineStr">
+        <is>
+          <t>B05-G013</t>
+        </is>
+      </c>
+      <c r="H221" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I221" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J221" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K221" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L221" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13331,27 +13731,47 @@
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E222" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F222" s="2" t="inlineStr"/>
-      <c r="G222" s="2" t="inlineStr"/>
-      <c r="H222" s="2" t="inlineStr"/>
-      <c r="I222" s="2" t="inlineStr"/>
-      <c r="J222" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G222" s="2" t="inlineStr">
+        <is>
+          <t>B05-G014; B05-G015; B05-G016</t>
+        </is>
+      </c>
+      <c r="H222" s="2" t="inlineStr">
+        <is>
+          <t>continuation_and_first_page</t>
+        </is>
+      </c>
+      <c r="I222" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J222" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K222" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_or_multi_instrument_extracted</t>
         </is>
       </c>
       <c r="L222" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13371,27 +13791,47 @@
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E223" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F223" s="2" t="inlineStr"/>
-      <c r="G223" s="2" t="inlineStr"/>
-      <c r="H223" s="2" t="inlineStr"/>
-      <c r="I223" s="2" t="inlineStr"/>
-      <c r="J223" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F223" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G223" s="2" t="inlineStr">
+        <is>
+          <t>B05-G016</t>
+        </is>
+      </c>
+      <c r="H223" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I223" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J223" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K223" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L223" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13411,27 +13851,47 @@
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E224" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F224" s="2" t="inlineStr"/>
-      <c r="G224" s="2" t="inlineStr"/>
-      <c r="H224" s="2" t="inlineStr"/>
-      <c r="I224" s="2" t="inlineStr"/>
-      <c r="J224" s="2" t="inlineStr"/>
+          <t>new_instrument_page</t>
+        </is>
+      </c>
+      <c r="F224" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G224" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H224" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I224" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J224" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K224" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L224" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13451,27 +13911,47 @@
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E225" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F225" s="2" t="inlineStr"/>
-      <c r="G225" s="2" t="inlineStr"/>
-      <c r="H225" s="2" t="inlineStr"/>
-      <c r="I225" s="2" t="inlineStr"/>
-      <c r="J225" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H225" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I225" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J225" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K225" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L225" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13491,27 +13971,47 @@
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E226" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F226" s="2" t="inlineStr"/>
-      <c r="G226" s="2" t="inlineStr"/>
-      <c r="H226" s="2" t="inlineStr"/>
-      <c r="I226" s="2" t="inlineStr"/>
-      <c r="J226" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G226" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H226" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I226" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J226" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K226" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L226" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13531,27 +14031,47 @@
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E227" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F227" s="2" t="inlineStr"/>
-      <c r="G227" s="2" t="inlineStr"/>
-      <c r="H227" s="2" t="inlineStr"/>
-      <c r="I227" s="2" t="inlineStr"/>
-      <c r="J227" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G227" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H227" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I227" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J227" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K227" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L227" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13571,27 +14091,47 @@
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E228" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F228" s="2" t="inlineStr"/>
-      <c r="G228" s="2" t="inlineStr"/>
-      <c r="H228" s="2" t="inlineStr"/>
-      <c r="I228" s="2" t="inlineStr"/>
-      <c r="J228" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G228" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H228" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I228" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J228" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K228" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L228" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13611,27 +14151,47 @@
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E229" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F229" s="2" t="inlineStr"/>
-      <c r="G229" s="2" t="inlineStr"/>
-      <c r="H229" s="2" t="inlineStr"/>
-      <c r="I229" s="2" t="inlineStr"/>
-      <c r="J229" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G229" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H229" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I229" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J229" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K229" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L229" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13651,27 +14211,47 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E230" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F230" s="2" t="inlineStr"/>
-      <c r="G230" s="2" t="inlineStr"/>
-      <c r="H230" s="2" t="inlineStr"/>
-      <c r="I230" s="2" t="inlineStr"/>
-      <c r="J230" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F230" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G230" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H230" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I230" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J230" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K230" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L230" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13691,27 +14271,47 @@
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E231" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F231" s="2" t="inlineStr"/>
-      <c r="G231" s="2" t="inlineStr"/>
-      <c r="H231" s="2" t="inlineStr"/>
-      <c r="I231" s="2" t="inlineStr"/>
-      <c r="J231" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F231" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G231" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H231" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I231" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J231" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K231" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L231" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13731,27 +14331,47 @@
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E232" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F232" s="2" t="inlineStr"/>
-      <c r="G232" s="2" t="inlineStr"/>
-      <c r="H232" s="2" t="inlineStr"/>
-      <c r="I232" s="2" t="inlineStr"/>
-      <c r="J232" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F232" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G232" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H232" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I232" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J232" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K232" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L232" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13771,27 +14391,47 @@
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E233" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F233" s="2" t="inlineStr"/>
-      <c r="G233" s="2" t="inlineStr"/>
-      <c r="H233" s="2" t="inlineStr"/>
-      <c r="I233" s="2" t="inlineStr"/>
-      <c r="J233" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F233" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G233" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H233" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I233" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J233" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K233" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L233" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13811,27 +14451,47 @@
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E234" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F234" s="2" t="inlineStr"/>
-      <c r="G234" s="2" t="inlineStr"/>
-      <c r="H234" s="2" t="inlineStr"/>
-      <c r="I234" s="2" t="inlineStr"/>
-      <c r="J234" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F234" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G234" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H234" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I234" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J234" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K234" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L234" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13851,27 +14511,47 @@
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E235" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F235" s="2" t="inlineStr"/>
-      <c r="G235" s="2" t="inlineStr"/>
-      <c r="H235" s="2" t="inlineStr"/>
-      <c r="I235" s="2" t="inlineStr"/>
-      <c r="J235" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F235" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G235" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H235" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I235" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J235" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K235" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L235" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13891,27 +14571,47 @@
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E236" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F236" s="2" t="inlineStr"/>
-      <c r="G236" s="2" t="inlineStr"/>
-      <c r="H236" s="2" t="inlineStr"/>
-      <c r="I236" s="2" t="inlineStr"/>
-      <c r="J236" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F236" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G236" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H236" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I236" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J236" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L236" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13931,27 +14631,47 @@
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E237" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F237" s="2" t="inlineStr"/>
-      <c r="G237" s="2" t="inlineStr"/>
-      <c r="H237" s="2" t="inlineStr"/>
-      <c r="I237" s="2" t="inlineStr"/>
-      <c r="J237" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F237" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G237" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H237" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I237" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J237" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K237" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L237" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -13971,27 +14691,47 @@
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E238" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F238" s="2" t="inlineStr"/>
-      <c r="G238" s="2" t="inlineStr"/>
-      <c r="H238" s="2" t="inlineStr"/>
-      <c r="I238" s="2" t="inlineStr"/>
-      <c r="J238" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G238" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H238" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I238" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J238" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K238" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L238" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -14011,27 +14751,47 @@
       </c>
       <c r="D239" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E239" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F239" s="2" t="inlineStr"/>
-      <c r="G239" s="2" t="inlineStr"/>
-      <c r="H239" s="2" t="inlineStr"/>
-      <c r="I239" s="2" t="inlineStr"/>
-      <c r="J239" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F239" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G239" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H239" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I239" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J239" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K239" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L239" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -14051,27 +14811,47 @@
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E240" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F240" s="2" t="inlineStr"/>
-      <c r="G240" s="2" t="inlineStr"/>
-      <c r="H240" s="2" t="inlineStr"/>
-      <c r="I240" s="2" t="inlineStr"/>
-      <c r="J240" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F240" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G240" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H240" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I240" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J240" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K240" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L240" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -14091,27 +14871,47 @@
       </c>
       <c r="D241" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E241" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F241" s="2" t="inlineStr"/>
-      <c r="G241" s="2" t="inlineStr"/>
-      <c r="H241" s="2" t="inlineStr"/>
-      <c r="I241" s="2" t="inlineStr"/>
-      <c r="J241" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F241" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G241" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H241" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I241" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J241" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K241" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L241" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -14131,27 +14931,47 @@
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E242" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F242" s="2" t="inlineStr"/>
-      <c r="G242" s="2" t="inlineStr"/>
-      <c r="H242" s="2" t="inlineStr"/>
-      <c r="I242" s="2" t="inlineStr"/>
-      <c r="J242" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G242" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H242" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I242" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J242" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K242" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L242" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -14171,27 +14991,47 @@
       </c>
       <c r="D243" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E243" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F243" s="2" t="inlineStr"/>
-      <c r="G243" s="2" t="inlineStr"/>
-      <c r="H243" s="2" t="inlineStr"/>
-      <c r="I243" s="2" t="inlineStr"/>
-      <c r="J243" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G243" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H243" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I243" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J243" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K243" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L243" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -14211,27 +15051,47 @@
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E244" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F244" s="2" t="inlineStr"/>
-      <c r="G244" s="2" t="inlineStr"/>
-      <c r="H244" s="2" t="inlineStr"/>
-      <c r="I244" s="2" t="inlineStr"/>
-      <c r="J244" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G244" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H244" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I244" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J244" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K244" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L244" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -14251,27 +15111,47 @@
       </c>
       <c r="D245" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E245" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F245" s="2" t="inlineStr"/>
-      <c r="G245" s="2" t="inlineStr"/>
-      <c r="H245" s="2" t="inlineStr"/>
-      <c r="I245" s="2" t="inlineStr"/>
-      <c r="J245" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G245" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H245" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I245" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J245" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K245" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L245" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -14291,27 +15171,47 @@
       </c>
       <c r="D246" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E246" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F246" s="2" t="inlineStr"/>
-      <c r="G246" s="2" t="inlineStr"/>
-      <c r="H246" s="2" t="inlineStr"/>
-      <c r="I246" s="2" t="inlineStr"/>
-      <c r="J246" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F246" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G246" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H246" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I246" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J246" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K246" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L246" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -14331,27 +15231,47 @@
       </c>
       <c r="D247" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E247" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F247" s="2" t="inlineStr"/>
-      <c r="G247" s="2" t="inlineStr"/>
-      <c r="H247" s="2" t="inlineStr"/>
-      <c r="I247" s="2" t="inlineStr"/>
-      <c r="J247" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G247" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H247" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I247" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J247" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K247" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L247" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -14371,27 +15291,47 @@
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E248" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F248" s="2" t="inlineStr"/>
-      <c r="G248" s="2" t="inlineStr"/>
-      <c r="H248" s="2" t="inlineStr"/>
-      <c r="I248" s="2" t="inlineStr"/>
-      <c r="J248" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H248" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I248" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J248" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K248" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L248" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -14411,27 +15351,47 @@
       </c>
       <c r="D249" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E249" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F249" s="2" t="inlineStr"/>
-      <c r="G249" s="2" t="inlineStr"/>
-      <c r="H249" s="2" t="inlineStr"/>
-      <c r="I249" s="2" t="inlineStr"/>
-      <c r="J249" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G249" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H249" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I249" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J249" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K249" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L249" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -14451,27 +15411,47 @@
       </c>
       <c r="D250" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E250" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F250" s="2" t="inlineStr"/>
-      <c r="G250" s="2" t="inlineStr"/>
-      <c r="H250" s="2" t="inlineStr"/>
-      <c r="I250" s="2" t="inlineStr"/>
-      <c r="J250" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G250" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H250" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I250" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J250" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K250" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L250" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -14491,27 +15471,47 @@
       </c>
       <c r="D251" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E251" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F251" s="2" t="inlineStr"/>
-      <c r="G251" s="2" t="inlineStr"/>
-      <c r="H251" s="2" t="inlineStr"/>
-      <c r="I251" s="2" t="inlineStr"/>
-      <c r="J251" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F251" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G251" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H251" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I251" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J251" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K251" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L251" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; zoom/enhancement and OCR were used only as aids. Stamps, signatures, marginal notes, legal schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Section 32 batch 06 checkpoint
Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
+++ b/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
@@ -15531,27 +15531,47 @@
       </c>
       <c r="D252" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E252" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F252" s="2" t="inlineStr"/>
-      <c r="G252" s="2" t="inlineStr"/>
-      <c r="H252" s="2" t="inlineStr"/>
-      <c r="I252" s="2" t="inlineStr"/>
-      <c r="J252" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G252" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H252" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I252" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J252" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K252" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L252" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -15571,27 +15591,47 @@
       </c>
       <c r="D253" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E253" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F253" s="2" t="inlineStr"/>
-      <c r="G253" s="2" t="inlineStr"/>
-      <c r="H253" s="2" t="inlineStr"/>
-      <c r="I253" s="2" t="inlineStr"/>
-      <c r="J253" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G253" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H253" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I253" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J253" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K253" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L253" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -15611,27 +15651,47 @@
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E254" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F254" s="2" t="inlineStr"/>
-      <c r="G254" s="2" t="inlineStr"/>
-      <c r="H254" s="2" t="inlineStr"/>
-      <c r="I254" s="2" t="inlineStr"/>
-      <c r="J254" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G254" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H254" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I254" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J254" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K254" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L254" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -15651,27 +15711,47 @@
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E255" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F255" s="2" t="inlineStr"/>
-      <c r="G255" s="2" t="inlineStr"/>
-      <c r="H255" s="2" t="inlineStr"/>
-      <c r="I255" s="2" t="inlineStr"/>
-      <c r="J255" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F255" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G255" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H255" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I255" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J255" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K255" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L255" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -15691,27 +15771,47 @@
       </c>
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E256" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F256" s="2" t="inlineStr"/>
-      <c r="G256" s="2" t="inlineStr"/>
-      <c r="H256" s="2" t="inlineStr"/>
-      <c r="I256" s="2" t="inlineStr"/>
-      <c r="J256" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G256" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H256" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I256" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J256" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K256" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L256" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -15731,27 +15831,47 @@
       </c>
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E257" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F257" s="2" t="inlineStr"/>
-      <c r="G257" s="2" t="inlineStr"/>
-      <c r="H257" s="2" t="inlineStr"/>
-      <c r="I257" s="2" t="inlineStr"/>
-      <c r="J257" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G257" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H257" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I257" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J257" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K257" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L257" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -15771,27 +15891,47 @@
       </c>
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E258" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F258" s="2" t="inlineStr"/>
-      <c r="G258" s="2" t="inlineStr"/>
-      <c r="H258" s="2" t="inlineStr"/>
-      <c r="I258" s="2" t="inlineStr"/>
-      <c r="J258" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G258" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H258" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I258" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J258" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K258" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L258" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -15811,27 +15951,47 @@
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E259" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F259" s="2" t="inlineStr"/>
-      <c r="G259" s="2" t="inlineStr"/>
-      <c r="H259" s="2" t="inlineStr"/>
-      <c r="I259" s="2" t="inlineStr"/>
-      <c r="J259" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F259" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G259" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H259" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I259" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J259" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K259" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L259" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -15851,27 +16011,47 @@
       </c>
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E260" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F260" s="2" t="inlineStr"/>
-      <c r="G260" s="2" t="inlineStr"/>
-      <c r="H260" s="2" t="inlineStr"/>
-      <c r="I260" s="2" t="inlineStr"/>
-      <c r="J260" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G260" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H260" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I260" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J260" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K260" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L260" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -15891,27 +16071,47 @@
       </c>
       <c r="D261" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E261" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F261" s="2" t="inlineStr"/>
-      <c r="G261" s="2" t="inlineStr"/>
-      <c r="H261" s="2" t="inlineStr"/>
-      <c r="I261" s="2" t="inlineStr"/>
-      <c r="J261" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F261" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G261" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H261" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I261" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J261" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K261" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L261" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -15931,27 +16131,47 @@
       </c>
       <c r="D262" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E262" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F262" s="2" t="inlineStr"/>
-      <c r="G262" s="2" t="inlineStr"/>
-      <c r="H262" s="2" t="inlineStr"/>
-      <c r="I262" s="2" t="inlineStr"/>
-      <c r="J262" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G262" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H262" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I262" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J262" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K262" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L262" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -15971,27 +16191,47 @@
       </c>
       <c r="D263" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E263" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F263" s="2" t="inlineStr"/>
-      <c r="G263" s="2" t="inlineStr"/>
-      <c r="H263" s="2" t="inlineStr"/>
-      <c r="I263" s="2" t="inlineStr"/>
-      <c r="J263" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G263" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H263" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I263" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J263" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K263" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L263" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16011,27 +16251,47 @@
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E264" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F264" s="2" t="inlineStr"/>
-      <c r="G264" s="2" t="inlineStr"/>
-      <c r="H264" s="2" t="inlineStr"/>
-      <c r="I264" s="2" t="inlineStr"/>
-      <c r="J264" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G264" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H264" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I264" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J264" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K264" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L264" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16051,27 +16311,47 @@
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E265" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F265" s="2" t="inlineStr"/>
-      <c r="G265" s="2" t="inlineStr"/>
-      <c r="H265" s="2" t="inlineStr"/>
-      <c r="I265" s="2" t="inlineStr"/>
-      <c r="J265" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F265" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G265" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H265" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I265" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J265" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K265" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L265" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16091,27 +16371,47 @@
       </c>
       <c r="D266" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E266" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F266" s="2" t="inlineStr"/>
-      <c r="G266" s="2" t="inlineStr"/>
-      <c r="H266" s="2" t="inlineStr"/>
-      <c r="I266" s="2" t="inlineStr"/>
-      <c r="J266" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F266" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G266" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H266" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I266" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J266" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K266" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L266" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16131,27 +16431,47 @@
       </c>
       <c r="D267" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E267" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F267" s="2" t="inlineStr"/>
-      <c r="G267" s="2" t="inlineStr"/>
-      <c r="H267" s="2" t="inlineStr"/>
-      <c r="I267" s="2" t="inlineStr"/>
-      <c r="J267" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F267" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G267" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H267" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I267" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J267" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K267" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L267" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16171,27 +16491,47 @@
       </c>
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E268" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F268" s="2" t="inlineStr"/>
-      <c r="G268" s="2" t="inlineStr"/>
-      <c r="H268" s="2" t="inlineStr"/>
-      <c r="I268" s="2" t="inlineStr"/>
-      <c r="J268" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F268" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G268" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H268" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I268" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J268" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K268" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L268" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16211,27 +16551,47 @@
       </c>
       <c r="D269" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E269" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F269" s="2" t="inlineStr"/>
-      <c r="G269" s="2" t="inlineStr"/>
-      <c r="H269" s="2" t="inlineStr"/>
-      <c r="I269" s="2" t="inlineStr"/>
-      <c r="J269" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F269" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G269" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H269" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I269" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J269" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K269" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L269" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16251,27 +16611,47 @@
       </c>
       <c r="D270" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E270" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F270" s="2" t="inlineStr"/>
-      <c r="G270" s="2" t="inlineStr"/>
-      <c r="H270" s="2" t="inlineStr"/>
-      <c r="I270" s="2" t="inlineStr"/>
-      <c r="J270" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F270" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G270" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H270" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I270" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J270" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K270" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L270" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16291,27 +16671,47 @@
       </c>
       <c r="D271" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E271" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F271" s="2" t="inlineStr"/>
-      <c r="G271" s="2" t="inlineStr"/>
-      <c r="H271" s="2" t="inlineStr"/>
-      <c r="I271" s="2" t="inlineStr"/>
-      <c r="J271" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F271" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G271" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H271" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I271" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J271" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K271" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L271" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16331,27 +16731,47 @@
       </c>
       <c r="D272" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E272" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F272" s="2" t="inlineStr"/>
-      <c r="G272" s="2" t="inlineStr"/>
-      <c r="H272" s="2" t="inlineStr"/>
-      <c r="I272" s="2" t="inlineStr"/>
-      <c r="J272" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G272" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H272" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I272" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J272" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K272" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L272" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16371,27 +16791,47 @@
       </c>
       <c r="D273" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E273" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F273" s="2" t="inlineStr"/>
-      <c r="G273" s="2" t="inlineStr"/>
-      <c r="H273" s="2" t="inlineStr"/>
-      <c r="I273" s="2" t="inlineStr"/>
-      <c r="J273" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F273" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G273" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H273" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I273" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J273" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K273" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L273" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16411,27 +16851,47 @@
       </c>
       <c r="D274" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E274" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F274" s="2" t="inlineStr"/>
-      <c r="G274" s="2" t="inlineStr"/>
-      <c r="H274" s="2" t="inlineStr"/>
-      <c r="I274" s="2" t="inlineStr"/>
-      <c r="J274" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F274" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G274" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H274" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I274" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J274" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K274" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L274" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16451,27 +16911,47 @@
       </c>
       <c r="D275" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E275" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F275" s="2" t="inlineStr"/>
-      <c r="G275" s="2" t="inlineStr"/>
-      <c r="H275" s="2" t="inlineStr"/>
-      <c r="I275" s="2" t="inlineStr"/>
-      <c r="J275" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F275" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G275" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H275" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I275" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J275" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K275" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L275" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16491,27 +16971,47 @@
       </c>
       <c r="D276" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E276" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F276" s="2" t="inlineStr"/>
-      <c r="G276" s="2" t="inlineStr"/>
-      <c r="H276" s="2" t="inlineStr"/>
-      <c r="I276" s="2" t="inlineStr"/>
-      <c r="J276" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F276" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G276" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H276" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I276" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J276" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K276" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L276" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16531,27 +17031,47 @@
       </c>
       <c r="D277" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E277" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F277" s="2" t="inlineStr"/>
-      <c r="G277" s="2" t="inlineStr"/>
-      <c r="H277" s="2" t="inlineStr"/>
-      <c r="I277" s="2" t="inlineStr"/>
-      <c r="J277" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F277" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G277" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H277" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I277" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J277" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K277" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L277" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16571,27 +17091,47 @@
       </c>
       <c r="D278" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E278" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F278" s="2" t="inlineStr"/>
-      <c r="G278" s="2" t="inlineStr"/>
-      <c r="H278" s="2" t="inlineStr"/>
-      <c r="I278" s="2" t="inlineStr"/>
-      <c r="J278" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F278" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G278" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H278" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I278" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J278" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K278" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L278" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16611,27 +17151,47 @@
       </c>
       <c r="D279" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E279" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F279" s="2" t="inlineStr"/>
-      <c r="G279" s="2" t="inlineStr"/>
-      <c r="H279" s="2" t="inlineStr"/>
-      <c r="I279" s="2" t="inlineStr"/>
-      <c r="J279" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F279" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G279" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H279" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I279" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J279" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K279" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L279" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16651,27 +17211,47 @@
       </c>
       <c r="D280" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E280" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F280" s="2" t="inlineStr"/>
-      <c r="G280" s="2" t="inlineStr"/>
-      <c r="H280" s="2" t="inlineStr"/>
-      <c r="I280" s="2" t="inlineStr"/>
-      <c r="J280" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F280" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G280" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H280" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I280" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J280" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K280" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L280" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16691,27 +17271,47 @@
       </c>
       <c r="D281" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E281" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F281" s="2" t="inlineStr"/>
-      <c r="G281" s="2" t="inlineStr"/>
-      <c r="H281" s="2" t="inlineStr"/>
-      <c r="I281" s="2" t="inlineStr"/>
-      <c r="J281" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F281" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G281" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H281" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I281" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J281" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K281" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L281" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16731,27 +17331,47 @@
       </c>
       <c r="D282" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E282" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F282" s="2" t="inlineStr"/>
-      <c r="G282" s="2" t="inlineStr"/>
-      <c r="H282" s="2" t="inlineStr"/>
-      <c r="I282" s="2" t="inlineStr"/>
-      <c r="J282" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F282" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G282" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H282" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I282" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J282" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K282" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L282" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16771,27 +17391,47 @@
       </c>
       <c r="D283" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E283" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F283" s="2" t="inlineStr"/>
-      <c r="G283" s="2" t="inlineStr"/>
-      <c r="H283" s="2" t="inlineStr"/>
-      <c r="I283" s="2" t="inlineStr"/>
-      <c r="J283" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F283" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G283" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H283" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I283" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J283" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K283" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L283" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16811,27 +17451,47 @@
       </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E284" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F284" s="2" t="inlineStr"/>
-      <c r="G284" s="2" t="inlineStr"/>
-      <c r="H284" s="2" t="inlineStr"/>
-      <c r="I284" s="2" t="inlineStr"/>
-      <c r="J284" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F284" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G284" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H284" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I284" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J284" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K284" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L284" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16851,27 +17511,47 @@
       </c>
       <c r="D285" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E285" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F285" s="2" t="inlineStr"/>
-      <c r="G285" s="2" t="inlineStr"/>
-      <c r="H285" s="2" t="inlineStr"/>
-      <c r="I285" s="2" t="inlineStr"/>
-      <c r="J285" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F285" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G285" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H285" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I285" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J285" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K285" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L285" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16891,27 +17571,47 @@
       </c>
       <c r="D286" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E286" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F286" s="2" t="inlineStr"/>
-      <c r="G286" s="2" t="inlineStr"/>
-      <c r="H286" s="2" t="inlineStr"/>
-      <c r="I286" s="2" t="inlineStr"/>
-      <c r="J286" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G286" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H286" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I286" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J286" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K286" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L286" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16931,27 +17631,47 @@
       </c>
       <c r="D287" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E287" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F287" s="2" t="inlineStr"/>
-      <c r="G287" s="2" t="inlineStr"/>
-      <c r="H287" s="2" t="inlineStr"/>
-      <c r="I287" s="2" t="inlineStr"/>
-      <c r="J287" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F287" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G287" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H287" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I287" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J287" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K287" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L287" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -16971,27 +17691,47 @@
       </c>
       <c r="D288" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E288" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F288" s="2" t="inlineStr"/>
-      <c r="G288" s="2" t="inlineStr"/>
-      <c r="H288" s="2" t="inlineStr"/>
-      <c r="I288" s="2" t="inlineStr"/>
-      <c r="J288" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F288" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G288" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H288" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I288" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J288" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K288" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L288" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -17011,27 +17751,47 @@
       </c>
       <c r="D289" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E289" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F289" s="2" t="inlineStr"/>
-      <c r="G289" s="2" t="inlineStr"/>
-      <c r="H289" s="2" t="inlineStr"/>
-      <c r="I289" s="2" t="inlineStr"/>
-      <c r="J289" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F289" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G289" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H289" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I289" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J289" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K289" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L289" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -17051,27 +17811,47 @@
       </c>
       <c r="D290" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E290" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F290" s="2" t="inlineStr"/>
-      <c r="G290" s="2" t="inlineStr"/>
-      <c r="H290" s="2" t="inlineStr"/>
-      <c r="I290" s="2" t="inlineStr"/>
-      <c r="J290" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F290" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G290" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H290" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I290" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J290" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K290" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L290" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -17091,27 +17871,47 @@
       </c>
       <c r="D291" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E291" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F291" s="2" t="inlineStr"/>
-      <c r="G291" s="2" t="inlineStr"/>
-      <c r="H291" s="2" t="inlineStr"/>
-      <c r="I291" s="2" t="inlineStr"/>
-      <c r="J291" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F291" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G291" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H291" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I291" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J291" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K291" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L291" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -17131,27 +17931,47 @@
       </c>
       <c r="D292" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E292" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F292" s="2" t="inlineStr"/>
-      <c r="G292" s="2" t="inlineStr"/>
-      <c r="H292" s="2" t="inlineStr"/>
-      <c r="I292" s="2" t="inlineStr"/>
-      <c r="J292" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F292" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G292" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H292" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I292" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J292" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K292" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L292" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -17171,27 +17991,47 @@
       </c>
       <c r="D293" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E293" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F293" s="2" t="inlineStr"/>
-      <c r="G293" s="2" t="inlineStr"/>
-      <c r="H293" s="2" t="inlineStr"/>
-      <c r="I293" s="2" t="inlineStr"/>
-      <c r="J293" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F293" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G293" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H293" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I293" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J293" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K293" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L293" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -17211,27 +18051,47 @@
       </c>
       <c r="D294" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E294" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F294" s="2" t="inlineStr"/>
-      <c r="G294" s="2" t="inlineStr"/>
-      <c r="H294" s="2" t="inlineStr"/>
-      <c r="I294" s="2" t="inlineStr"/>
-      <c r="J294" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F294" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G294" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H294" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I294" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J294" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K294" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L294" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -17251,27 +18111,47 @@
       </c>
       <c r="D295" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E295" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F295" s="2" t="inlineStr"/>
-      <c r="G295" s="2" t="inlineStr"/>
-      <c r="H295" s="2" t="inlineStr"/>
-      <c r="I295" s="2" t="inlineStr"/>
-      <c r="J295" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F295" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G295" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H295" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I295" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J295" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K295" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L295" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -17291,27 +18171,47 @@
       </c>
       <c r="D296" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E296" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F296" s="2" t="inlineStr"/>
-      <c r="G296" s="2" t="inlineStr"/>
-      <c r="H296" s="2" t="inlineStr"/>
-      <c r="I296" s="2" t="inlineStr"/>
-      <c r="J296" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F296" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G296" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H296" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I296" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J296" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K296" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L296" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -17331,27 +18231,47 @@
       </c>
       <c r="D297" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E297" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F297" s="2" t="inlineStr"/>
-      <c r="G297" s="2" t="inlineStr"/>
-      <c r="H297" s="2" t="inlineStr"/>
-      <c r="I297" s="2" t="inlineStr"/>
-      <c r="J297" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F297" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G297" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H297" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I297" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J297" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K297" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L297" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -17371,27 +18291,47 @@
       </c>
       <c r="D298" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E298" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F298" s="2" t="inlineStr"/>
-      <c r="G298" s="2" t="inlineStr"/>
-      <c r="H298" s="2" t="inlineStr"/>
-      <c r="I298" s="2" t="inlineStr"/>
-      <c r="J298" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F298" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G298" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H298" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I298" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J298" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K298" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L298" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -17411,27 +18351,47 @@
       </c>
       <c r="D299" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E299" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F299" s="2" t="inlineStr"/>
-      <c r="G299" s="2" t="inlineStr"/>
-      <c r="H299" s="2" t="inlineStr"/>
-      <c r="I299" s="2" t="inlineStr"/>
-      <c r="J299" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F299" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G299" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H299" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I299" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J299" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K299" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L299" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -17451,27 +18411,47 @@
       </c>
       <c r="D300" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E300" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F300" s="2" t="inlineStr"/>
-      <c r="G300" s="2" t="inlineStr"/>
-      <c r="H300" s="2" t="inlineStr"/>
-      <c r="I300" s="2" t="inlineStr"/>
-      <c r="J300" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F300" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G300" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H300" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I300" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J300" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K300" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L300" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>
@@ -17491,27 +18471,47 @@
       </c>
       <c r="D301" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E301" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F301" s="2" t="inlineStr"/>
-      <c r="G301" s="2" t="inlineStr"/>
-      <c r="H301" s="2" t="inlineStr"/>
-      <c r="I301" s="2" t="inlineStr"/>
-      <c r="J301" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F301" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G301" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H301" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I301" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J301" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K301" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L301" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at page scale; stamps, signatures, marginal notes, schedules, and continuity were checked. This page continues the same recorded indenture; no separate instrument begins on the page.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Section 32 batch 07 checkpoint
Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
+++ b/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
@@ -18531,27 +18531,47 @@
       </c>
       <c r="D302" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E302" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F302" s="2" t="inlineStr"/>
-      <c r="G302" s="2" t="inlineStr"/>
-      <c r="H302" s="2" t="inlineStr"/>
-      <c r="I302" s="2" t="inlineStr"/>
-      <c r="J302" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F302" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G302" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H302" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I302" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J302" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K302" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L302" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -18571,27 +18591,47 @@
       </c>
       <c r="D303" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E303" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F303" s="2" t="inlineStr"/>
-      <c r="G303" s="2" t="inlineStr"/>
-      <c r="H303" s="2" t="inlineStr"/>
-      <c r="I303" s="2" t="inlineStr"/>
-      <c r="J303" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F303" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G303" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H303" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I303" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J303" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K303" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L303" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -18611,27 +18651,47 @@
       </c>
       <c r="D304" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E304" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F304" s="2" t="inlineStr"/>
-      <c r="G304" s="2" t="inlineStr"/>
-      <c r="H304" s="2" t="inlineStr"/>
-      <c r="I304" s="2" t="inlineStr"/>
-      <c r="J304" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F304" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G304" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H304" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I304" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J304" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K304" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L304" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -18651,27 +18711,47 @@
       </c>
       <c r="D305" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E305" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F305" s="2" t="inlineStr"/>
-      <c r="G305" s="2" t="inlineStr"/>
-      <c r="H305" s="2" t="inlineStr"/>
-      <c r="I305" s="2" t="inlineStr"/>
-      <c r="J305" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F305" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G305" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H305" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I305" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J305" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K305" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L305" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -18691,27 +18771,47 @@
       </c>
       <c r="D306" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E306" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F306" s="2" t="inlineStr"/>
-      <c r="G306" s="2" t="inlineStr"/>
-      <c r="H306" s="2" t="inlineStr"/>
-      <c r="I306" s="2" t="inlineStr"/>
-      <c r="J306" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F306" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G306" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H306" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I306" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J306" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K306" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L306" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -18731,27 +18831,47 @@
       </c>
       <c r="D307" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E307" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F307" s="2" t="inlineStr"/>
-      <c r="G307" s="2" t="inlineStr"/>
-      <c r="H307" s="2" t="inlineStr"/>
-      <c r="I307" s="2" t="inlineStr"/>
-      <c r="J307" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F307" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G307" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H307" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I307" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J307" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K307" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L307" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -18771,27 +18891,47 @@
       </c>
       <c r="D308" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E308" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F308" s="2" t="inlineStr"/>
-      <c r="G308" s="2" t="inlineStr"/>
-      <c r="H308" s="2" t="inlineStr"/>
-      <c r="I308" s="2" t="inlineStr"/>
-      <c r="J308" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F308" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G308" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H308" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I308" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J308" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K308" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L308" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -18811,27 +18951,47 @@
       </c>
       <c r="D309" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E309" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F309" s="2" t="inlineStr"/>
-      <c r="G309" s="2" t="inlineStr"/>
-      <c r="H309" s="2" t="inlineStr"/>
-      <c r="I309" s="2" t="inlineStr"/>
-      <c r="J309" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F309" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G309" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H309" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I309" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J309" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K309" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L309" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -18851,27 +19011,47 @@
       </c>
       <c r="D310" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E310" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F310" s="2" t="inlineStr"/>
-      <c r="G310" s="2" t="inlineStr"/>
-      <c r="H310" s="2" t="inlineStr"/>
-      <c r="I310" s="2" t="inlineStr"/>
-      <c r="J310" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F310" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G310" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H310" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I310" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J310" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K310" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L310" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -18891,27 +19071,47 @@
       </c>
       <c r="D311" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E311" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F311" s="2" t="inlineStr"/>
-      <c r="G311" s="2" t="inlineStr"/>
-      <c r="H311" s="2" t="inlineStr"/>
-      <c r="I311" s="2" t="inlineStr"/>
-      <c r="J311" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F311" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G311" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H311" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I311" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J311" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K311" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L311" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -18931,27 +19131,47 @@
       </c>
       <c r="D312" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E312" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F312" s="2" t="inlineStr"/>
-      <c r="G312" s="2" t="inlineStr"/>
-      <c r="H312" s="2" t="inlineStr"/>
-      <c r="I312" s="2" t="inlineStr"/>
-      <c r="J312" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F312" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G312" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H312" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I312" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J312" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K312" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L312" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -18971,27 +19191,47 @@
       </c>
       <c r="D313" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E313" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F313" s="2" t="inlineStr"/>
-      <c r="G313" s="2" t="inlineStr"/>
-      <c r="H313" s="2" t="inlineStr"/>
-      <c r="I313" s="2" t="inlineStr"/>
-      <c r="J313" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F313" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G313" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H313" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I313" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J313" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K313" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L313" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19011,27 +19251,47 @@
       </c>
       <c r="D314" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E314" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F314" s="2" t="inlineStr"/>
-      <c r="G314" s="2" t="inlineStr"/>
-      <c r="H314" s="2" t="inlineStr"/>
-      <c r="I314" s="2" t="inlineStr"/>
-      <c r="J314" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F314" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G314" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H314" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I314" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J314" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K314" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L314" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19051,27 +19311,47 @@
       </c>
       <c r="D315" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E315" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F315" s="2" t="inlineStr"/>
-      <c r="G315" s="2" t="inlineStr"/>
-      <c r="H315" s="2" t="inlineStr"/>
-      <c r="I315" s="2" t="inlineStr"/>
-      <c r="J315" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F315" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G315" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H315" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I315" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J315" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K315" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L315" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19091,27 +19371,47 @@
       </c>
       <c r="D316" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E316" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F316" s="2" t="inlineStr"/>
-      <c r="G316" s="2" t="inlineStr"/>
-      <c r="H316" s="2" t="inlineStr"/>
-      <c r="I316" s="2" t="inlineStr"/>
-      <c r="J316" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F316" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G316" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H316" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I316" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J316" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K316" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L316" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19131,27 +19431,47 @@
       </c>
       <c r="D317" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E317" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F317" s="2" t="inlineStr"/>
-      <c r="G317" s="2" t="inlineStr"/>
-      <c r="H317" s="2" t="inlineStr"/>
-      <c r="I317" s="2" t="inlineStr"/>
-      <c r="J317" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F317" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G317" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H317" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I317" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J317" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K317" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L317" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19171,27 +19491,47 @@
       </c>
       <c r="D318" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E318" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F318" s="2" t="inlineStr"/>
-      <c r="G318" s="2" t="inlineStr"/>
-      <c r="H318" s="2" t="inlineStr"/>
-      <c r="I318" s="2" t="inlineStr"/>
-      <c r="J318" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F318" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G318" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H318" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I318" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J318" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K318" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L318" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19211,27 +19551,47 @@
       </c>
       <c r="D319" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E319" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F319" s="2" t="inlineStr"/>
-      <c r="G319" s="2" t="inlineStr"/>
-      <c r="H319" s="2" t="inlineStr"/>
-      <c r="I319" s="2" t="inlineStr"/>
-      <c r="J319" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F319" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G319" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H319" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I319" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J319" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K319" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L319" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19251,27 +19611,47 @@
       </c>
       <c r="D320" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E320" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F320" s="2" t="inlineStr"/>
-      <c r="G320" s="2" t="inlineStr"/>
-      <c r="H320" s="2" t="inlineStr"/>
-      <c r="I320" s="2" t="inlineStr"/>
-      <c r="J320" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F320" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G320" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H320" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I320" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J320" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K320" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L320" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19291,27 +19671,47 @@
       </c>
       <c r="D321" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E321" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F321" s="2" t="inlineStr"/>
-      <c r="G321" s="2" t="inlineStr"/>
-      <c r="H321" s="2" t="inlineStr"/>
-      <c r="I321" s="2" t="inlineStr"/>
-      <c r="J321" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F321" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G321" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H321" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I321" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J321" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K321" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L321" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19331,27 +19731,47 @@
       </c>
       <c r="D322" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E322" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F322" s="2" t="inlineStr"/>
-      <c r="G322" s="2" t="inlineStr"/>
-      <c r="H322" s="2" t="inlineStr"/>
-      <c r="I322" s="2" t="inlineStr"/>
-      <c r="J322" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F322" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G322" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H322" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I322" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J322" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K322" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L322" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19371,27 +19791,47 @@
       </c>
       <c r="D323" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E323" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F323" s="2" t="inlineStr"/>
-      <c r="G323" s="2" t="inlineStr"/>
-      <c r="H323" s="2" t="inlineStr"/>
-      <c r="I323" s="2" t="inlineStr"/>
-      <c r="J323" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F323" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G323" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H323" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I323" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J323" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K323" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L323" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19411,27 +19851,47 @@
       </c>
       <c r="D324" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E324" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F324" s="2" t="inlineStr"/>
-      <c r="G324" s="2" t="inlineStr"/>
-      <c r="H324" s="2" t="inlineStr"/>
-      <c r="I324" s="2" t="inlineStr"/>
-      <c r="J324" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F324" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G324" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H324" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I324" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J324" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K324" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L324" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19451,27 +19911,47 @@
       </c>
       <c r="D325" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E325" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F325" s="2" t="inlineStr"/>
-      <c r="G325" s="2" t="inlineStr"/>
-      <c r="H325" s="2" t="inlineStr"/>
-      <c r="I325" s="2" t="inlineStr"/>
-      <c r="J325" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F325" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G325" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H325" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I325" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J325" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K325" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L325" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19491,27 +19971,47 @@
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E326" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F326" s="2" t="inlineStr"/>
-      <c r="G326" s="2" t="inlineStr"/>
-      <c r="H326" s="2" t="inlineStr"/>
-      <c r="I326" s="2" t="inlineStr"/>
-      <c r="J326" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F326" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G326" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H326" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I326" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J326" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K326" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L326" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19531,27 +20031,47 @@
       </c>
       <c r="D327" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E327" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F327" s="2" t="inlineStr"/>
-      <c r="G327" s="2" t="inlineStr"/>
-      <c r="H327" s="2" t="inlineStr"/>
-      <c r="I327" s="2" t="inlineStr"/>
-      <c r="J327" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F327" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G327" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H327" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I327" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J327" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K327" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L327" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19571,27 +20091,47 @@
       </c>
       <c r="D328" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E328" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F328" s="2" t="inlineStr"/>
-      <c r="G328" s="2" t="inlineStr"/>
-      <c r="H328" s="2" t="inlineStr"/>
-      <c r="I328" s="2" t="inlineStr"/>
-      <c r="J328" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F328" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G328" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H328" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I328" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J328" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K328" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L328" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19611,27 +20151,47 @@
       </c>
       <c r="D329" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E329" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F329" s="2" t="inlineStr"/>
-      <c r="G329" s="2" t="inlineStr"/>
-      <c r="H329" s="2" t="inlineStr"/>
-      <c r="I329" s="2" t="inlineStr"/>
-      <c r="J329" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F329" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G329" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H329" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I329" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J329" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19651,27 +20211,47 @@
       </c>
       <c r="D330" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E330" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F330" s="2" t="inlineStr"/>
-      <c r="G330" s="2" t="inlineStr"/>
-      <c r="H330" s="2" t="inlineStr"/>
-      <c r="I330" s="2" t="inlineStr"/>
-      <c r="J330" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F330" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G330" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H330" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I330" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J330" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the 1941 indenture without a separate instrument.</t>
         </is>
       </c>
     </row>
@@ -19691,27 +20271,47 @@
       </c>
       <c r="D331" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E331" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F331" s="2" t="inlineStr"/>
-      <c r="G331" s="2" t="inlineStr"/>
-      <c r="H331" s="2" t="inlineStr"/>
-      <c r="I331" s="2" t="inlineStr"/>
-      <c r="J331" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F331" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G331" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H331" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I331" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J331" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Execution, signatures, seals, multistate acknowledgment forms, and the final recorder certification were inspected.</t>
         </is>
       </c>
     </row>
@@ -19731,27 +20331,47 @@
       </c>
       <c r="D332" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E332" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F332" s="2" t="inlineStr"/>
-      <c r="G332" s="2" t="inlineStr"/>
-      <c r="H332" s="2" t="inlineStr"/>
-      <c r="I332" s="2" t="inlineStr"/>
-      <c r="J332" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F332" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G332" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H332" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I332" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J332" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K332" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L332" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Execution, signatures, seals, multistate acknowledgment forms, and the final recorder certification were inspected.</t>
         </is>
       </c>
     </row>
@@ -19771,27 +20391,47 @@
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E333" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F333" s="2" t="inlineStr"/>
-      <c r="G333" s="2" t="inlineStr"/>
-      <c r="H333" s="2" t="inlineStr"/>
-      <c r="I333" s="2" t="inlineStr"/>
-      <c r="J333" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F333" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G333" s="2" t="inlineStr">
+        <is>
+          <t>B05-G017</t>
+        </is>
+      </c>
+      <c r="H333" s="2" t="inlineStr">
+        <is>
+          <t>final_page</t>
+        </is>
+      </c>
+      <c r="I333" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J333" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K333" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L333" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Execution, signatures, seals, multistate acknowledgment forms, and the final recorder certification were inspected.</t>
         </is>
       </c>
     </row>
@@ -19811,27 +20451,47 @@
       </c>
       <c r="D334" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E334" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F334" s="2" t="inlineStr"/>
-      <c r="G334" s="2" t="inlineStr"/>
-      <c r="H334" s="2" t="inlineStr"/>
-      <c r="I334" s="2" t="inlineStr"/>
-      <c r="J334" s="2" t="inlineStr"/>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="F334" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G334" s="2" t="inlineStr">
+        <is>
+          <t>B07-G001</t>
+        </is>
+      </c>
+      <c r="H334" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I334" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J334" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K334" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L334" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. General release of the 1928 mortgage and its supplements; recording schedules, signatures, seals, and acknowledgments were inspected.</t>
         </is>
       </c>
     </row>
@@ -19851,27 +20511,47 @@
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E335" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F335" s="2" t="inlineStr"/>
-      <c r="G335" s="2" t="inlineStr"/>
-      <c r="H335" s="2" t="inlineStr"/>
-      <c r="I335" s="2" t="inlineStr"/>
-      <c r="J335" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F335" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G335" s="2" t="inlineStr">
+        <is>
+          <t>B07-G001</t>
+        </is>
+      </c>
+      <c r="H335" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I335" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J335" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K335" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L335" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. General release of the 1928 mortgage and its supplements; recording schedules, signatures, seals, and acknowledgments were inspected.</t>
         </is>
       </c>
     </row>
@@ -19891,27 +20571,47 @@
       </c>
       <c r="D336" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E336" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F336" s="2" t="inlineStr"/>
-      <c r="G336" s="2" t="inlineStr"/>
-      <c r="H336" s="2" t="inlineStr"/>
-      <c r="I336" s="2" t="inlineStr"/>
-      <c r="J336" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F336" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G336" s="2" t="inlineStr">
+        <is>
+          <t>B07-G001</t>
+        </is>
+      </c>
+      <c r="H336" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I336" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J336" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K336" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L336" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. General release of the 1928 mortgage and its supplements; recording schedules, signatures, seals, and acknowledgments were inspected.</t>
         </is>
       </c>
     </row>
@@ -19931,27 +20631,47 @@
       </c>
       <c r="D337" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E337" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F337" s="2" t="inlineStr"/>
-      <c r="G337" s="2" t="inlineStr"/>
-      <c r="H337" s="2" t="inlineStr"/>
-      <c r="I337" s="2" t="inlineStr"/>
-      <c r="J337" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F337" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G337" s="2" t="inlineStr">
+        <is>
+          <t>B07-G001</t>
+        </is>
+      </c>
+      <c r="H337" s="2" t="inlineStr">
+        <is>
+          <t>final_page</t>
+        </is>
+      </c>
+      <c r="I337" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J337" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K337" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L337" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. General release of the 1928 mortgage and its supplements; recording schedules, signatures, seals, and acknowledgments were inspected.</t>
         </is>
       </c>
     </row>
@@ -19971,27 +20691,47 @@
       </c>
       <c r="D338" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E338" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F338" s="2" t="inlineStr"/>
-      <c r="G338" s="2" t="inlineStr"/>
-      <c r="H338" s="2" t="inlineStr"/>
-      <c r="I338" s="2" t="inlineStr"/>
-      <c r="J338" s="2" t="inlineStr"/>
+          <t>single_page_instrument</t>
+        </is>
+      </c>
+      <c r="F338" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G338" s="2" t="inlineStr">
+        <is>
+          <t>B07-G002</t>
+        </is>
+      </c>
+      <c r="H338" s="2" t="inlineStr">
+        <is>
+          <t>first_and_final_page</t>
+        </is>
+      </c>
+      <c r="I338" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J338" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K338" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L338" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Single-page quitclaim deed; typed legal calls, execution, acknowledgment, and filing stamp were inspected.</t>
         </is>
       </c>
     </row>
@@ -20011,27 +20751,47 @@
       </c>
       <c r="D339" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E339" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F339" s="2" t="inlineStr"/>
-      <c r="G339" s="2" t="inlineStr"/>
-      <c r="H339" s="2" t="inlineStr"/>
-      <c r="I339" s="2" t="inlineStr"/>
-      <c r="J339" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F339" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G339" s="2" t="inlineStr">
+        <is>
+          <t>B07-G003; B07-G004</t>
+        </is>
+      </c>
+      <c r="H339" s="2" t="inlineStr">
+        <is>
+          <t>mixed_final_and_first_page</t>
+        </is>
+      </c>
+      <c r="I339" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J339" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K339" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L339" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. The page ends an otherwise unavailable M. M. Bennett mortgage and begins the Keathley mortgage; both instruments were split.</t>
         </is>
       </c>
     </row>
@@ -20051,27 +20811,47 @@
       </c>
       <c r="D340" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E340" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F340" s="2" t="inlineStr"/>
-      <c r="G340" s="2" t="inlineStr"/>
-      <c r="H340" s="2" t="inlineStr"/>
-      <c r="I340" s="2" t="inlineStr"/>
-      <c r="J340" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F340" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G340" s="2" t="inlineStr">
+        <is>
+          <t>B07-G004</t>
+        </is>
+      </c>
+      <c r="H340" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I340" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J340" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K340" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L340" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Keathley mortgage continuation containing the Section 32 legal description and secured-debt terms.</t>
         </is>
       </c>
     </row>
@@ -20091,27 +20871,47 @@
       </c>
       <c r="D341" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E341" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F341" s="2" t="inlineStr"/>
-      <c r="G341" s="2" t="inlineStr"/>
-      <c r="H341" s="2" t="inlineStr"/>
-      <c r="I341" s="2" t="inlineStr"/>
-      <c r="J341" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F341" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G341" s="2" t="inlineStr">
+        <is>
+          <t>B07-G004; B07-G005</t>
+        </is>
+      </c>
+      <c r="H341" s="2" t="inlineStr">
+        <is>
+          <t>mixed_final_and_first_page</t>
+        </is>
+      </c>
+      <c r="I341" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J341" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K341" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L341" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. The Keathley mortgage ends with signatures and acknowledgment; a separate Prock mortgage begins and was split.</t>
         </is>
       </c>
     </row>
@@ -20131,27 +20931,47 @@
       </c>
       <c r="D342" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E342" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F342" s="2" t="inlineStr"/>
-      <c r="G342" s="2" t="inlineStr"/>
-      <c r="H342" s="2" t="inlineStr"/>
-      <c r="I342" s="2" t="inlineStr"/>
-      <c r="J342" s="2" t="inlineStr"/>
+          <t>single_page_instrument</t>
+        </is>
+      </c>
+      <c r="F342" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G342" s="2" t="inlineStr">
+        <is>
+          <t>B07-G006</t>
+        </is>
+      </c>
+      <c r="H342" s="2" t="inlineStr">
+        <is>
+          <t>first_and_final_page</t>
+        </is>
+      </c>
+      <c r="I342" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J342" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Single-page warranty deed; parties, exact aliquot calls, acreage, signatures, acknowledgment, and filing data were inspected.</t>
         </is>
       </c>
     </row>
@@ -20171,27 +20991,47 @@
       </c>
       <c r="D343" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E343" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F343" s="2" t="inlineStr"/>
-      <c r="G343" s="2" t="inlineStr"/>
-      <c r="H343" s="2" t="inlineStr"/>
-      <c r="I343" s="2" t="inlineStr"/>
-      <c r="J343" s="2" t="inlineStr"/>
+          <t>single_page_instrument</t>
+        </is>
+      </c>
+      <c r="F343" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G343" s="2" t="inlineStr">
+        <is>
+          <t>B07-G007</t>
+        </is>
+      </c>
+      <c r="H343" s="2" t="inlineStr">
+        <is>
+          <t>first_and_final_page</t>
+        </is>
+      </c>
+      <c r="I343" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J343" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K343" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L343" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Single-page warranty deed; parties, exact aliquot calls, acreage, signatures, acknowledgment, and filing data were inspected.</t>
         </is>
       </c>
     </row>
@@ -20211,27 +21051,47 @@
       </c>
       <c r="D344" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E344" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F344" s="2" t="inlineStr"/>
-      <c r="G344" s="2" t="inlineStr"/>
-      <c r="H344" s="2" t="inlineStr"/>
-      <c r="I344" s="2" t="inlineStr"/>
-      <c r="J344" s="2" t="inlineStr"/>
+          <t>single_page_instrument</t>
+        </is>
+      </c>
+      <c r="F344" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G344" s="2" t="inlineStr">
+        <is>
+          <t>B07-G008</t>
+        </is>
+      </c>
+      <c r="H344" s="2" t="inlineStr">
+        <is>
+          <t>first_and_final_page</t>
+        </is>
+      </c>
+      <c r="I344" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J344" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K344" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L344" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Single-page warranty deed; parties, exact aliquot calls, acreage, signatures, acknowledgment, and filing data were inspected.</t>
         </is>
       </c>
     </row>
@@ -20251,27 +21111,47 @@
       </c>
       <c r="D345" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E345" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F345" s="2" t="inlineStr"/>
-      <c r="G345" s="2" t="inlineStr"/>
-      <c r="H345" s="2" t="inlineStr"/>
-      <c r="I345" s="2" t="inlineStr"/>
-      <c r="J345" s="2" t="inlineStr"/>
+          <t>single_page_instrument</t>
+        </is>
+      </c>
+      <c r="F345" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G345" s="2" t="inlineStr">
+        <is>
+          <t>B07-G009</t>
+        </is>
+      </c>
+      <c r="H345" s="2" t="inlineStr">
+        <is>
+          <t>first_and_final_page</t>
+        </is>
+      </c>
+      <c r="I345" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J345" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K345" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L345" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Single-page warranty deed; parties, exact aliquot calls, acreage, signatures, acknowledgment, and filing data were inspected.</t>
         </is>
       </c>
     </row>
@@ -20291,27 +21171,47 @@
       </c>
       <c r="D346" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E346" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F346" s="2" t="inlineStr"/>
-      <c r="G346" s="2" t="inlineStr"/>
-      <c r="H346" s="2" t="inlineStr"/>
-      <c r="I346" s="2" t="inlineStr"/>
-      <c r="J346" s="2" t="inlineStr"/>
+          <t>single_page_instrument</t>
+        </is>
+      </c>
+      <c r="F346" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G346" s="2" t="inlineStr">
+        <is>
+          <t>B07-G010</t>
+        </is>
+      </c>
+      <c r="H346" s="2" t="inlineStr">
+        <is>
+          <t>first_and_final_page</t>
+        </is>
+      </c>
+      <c r="I346" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J346" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K346" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L346" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Single-page warranty deed; parties, exact aliquot calls, acreage, signatures, acknowledgment, and filing data were inspected.</t>
         </is>
       </c>
     </row>
@@ -20331,27 +21231,47 @@
       </c>
       <c r="D347" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E347" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F347" s="2" t="inlineStr"/>
-      <c r="G347" s="2" t="inlineStr"/>
-      <c r="H347" s="2" t="inlineStr"/>
-      <c r="I347" s="2" t="inlineStr"/>
-      <c r="J347" s="2" t="inlineStr"/>
+          <t>single_page_instrument</t>
+        </is>
+      </c>
+      <c r="F347" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G347" s="2" t="inlineStr">
+        <is>
+          <t>B07-G011</t>
+        </is>
+      </c>
+      <c r="H347" s="2" t="inlineStr">
+        <is>
+          <t>first_and_final_page</t>
+        </is>
+      </c>
+      <c r="I347" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J347" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K347" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L347" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Single-page warranty deed; parties, exact aliquot calls, acreage, signatures, acknowledgment, and filing data were inspected.</t>
         </is>
       </c>
     </row>
@@ -20371,27 +21291,47 @@
       </c>
       <c r="D348" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E348" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F348" s="2" t="inlineStr"/>
-      <c r="G348" s="2" t="inlineStr"/>
-      <c r="H348" s="2" t="inlineStr"/>
-      <c r="I348" s="2" t="inlineStr"/>
-      <c r="J348" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F348" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G348" s="2" t="inlineStr">
+        <is>
+          <t>B07-G012; B07-G013</t>
+        </is>
+      </c>
+      <c r="H348" s="2" t="inlineStr">
+        <is>
+          <t>mixed_single_and_first_page</t>
+        </is>
+      </c>
+      <c r="I348" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J348" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K348" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L348" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. A complete unrelated oil-and-gas-lease release occupies the top; the general release of the 1941 indenture begins below and was split.</t>
         </is>
       </c>
     </row>
@@ -20411,27 +21351,47 @@
       </c>
       <c r="D349" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E349" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F349" s="2" t="inlineStr"/>
-      <c r="G349" s="2" t="inlineStr"/>
-      <c r="H349" s="2" t="inlineStr"/>
-      <c r="I349" s="2" t="inlineStr"/>
-      <c r="J349" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F349" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G349" s="2" t="inlineStr">
+        <is>
+          <t>B07-G013</t>
+        </is>
+      </c>
+      <c r="H349" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I349" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J349" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K349" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L349" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the general release through mortgage/chattel-mortgage schedules; page 0351 was checked only for the ending.</t>
         </is>
       </c>
     </row>
@@ -20451,27 +21411,47 @@
       </c>
       <c r="D350" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E350" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F350" s="2" t="inlineStr"/>
-      <c r="G350" s="2" t="inlineStr"/>
-      <c r="H350" s="2" t="inlineStr"/>
-      <c r="I350" s="2" t="inlineStr"/>
-      <c r="J350" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F350" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G350" s="2" t="inlineStr">
+        <is>
+          <t>B07-G013</t>
+        </is>
+      </c>
+      <c r="H350" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I350" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J350" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K350" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L350" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the general release through mortgage/chattel-mortgage schedules; page 0351 was checked only for the ending.</t>
         </is>
       </c>
     </row>
@@ -20491,27 +21471,47 @@
       </c>
       <c r="D351" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E351" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F351" s="2" t="inlineStr"/>
-      <c r="G351" s="2" t="inlineStr"/>
-      <c r="H351" s="2" t="inlineStr"/>
-      <c r="I351" s="2" t="inlineStr"/>
-      <c r="J351" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F351" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G351" s="2" t="inlineStr">
+        <is>
+          <t>B07-G013</t>
+        </is>
+      </c>
+      <c r="H351" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I351" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J351" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K351" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L351" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly; page continuity, marginal notes, stamps, signatures, seals, schedules, and legal calls were checked. Continues the general release through mortgage/chattel-mortgage schedules; page 0351 was checked only for the ending.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Section 32 batch 08 checkpoint
Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
+++ b/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
@@ -21531,27 +21531,47 @@
       </c>
       <c r="D352" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E352" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F352" s="2" t="inlineStr"/>
-      <c r="G352" s="2" t="inlineStr"/>
-      <c r="H352" s="2" t="inlineStr"/>
-      <c r="I352" s="2" t="inlineStr"/>
-      <c r="J352" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F352" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G352" s="2" t="inlineStr">
+        <is>
+          <t>B07-G013</t>
+        </is>
+      </c>
+      <c r="H352" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I352" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J352" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K352" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L352" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -21571,27 +21591,47 @@
       </c>
       <c r="D353" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E353" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F353" s="2" t="inlineStr"/>
-      <c r="G353" s="2" t="inlineStr"/>
-      <c r="H353" s="2" t="inlineStr"/>
-      <c r="I353" s="2" t="inlineStr"/>
-      <c r="J353" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F353" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G353" s="2" t="inlineStr">
+        <is>
+          <t>B08-G001; B08-G002</t>
+        </is>
+      </c>
+      <c r="H353" s="2" t="inlineStr">
+        <is>
+          <t>multiple_single_page_instruments</t>
+        </is>
+      </c>
+      <c r="I353" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J353" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K353" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L353" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -21611,27 +21651,47 @@
       </c>
       <c r="D354" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E354" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F354" s="2" t="inlineStr"/>
-      <c r="G354" s="2" t="inlineStr"/>
-      <c r="H354" s="2" t="inlineStr"/>
-      <c r="I354" s="2" t="inlineStr"/>
-      <c r="J354" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F354" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G354" s="2" t="inlineStr">
+        <is>
+          <t>B08-G003</t>
+        </is>
+      </c>
+      <c r="H354" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I354" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J354" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K354" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L354" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -21651,27 +21711,47 @@
       </c>
       <c r="D355" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E355" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F355" s="2" t="inlineStr"/>
-      <c r="G355" s="2" t="inlineStr"/>
-      <c r="H355" s="2" t="inlineStr"/>
-      <c r="I355" s="2" t="inlineStr"/>
-      <c r="J355" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F355" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G355" s="2" t="inlineStr">
+        <is>
+          <t>B08-G004</t>
+        </is>
+      </c>
+      <c r="H355" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I355" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J355" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K355" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L355" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -21691,27 +21771,47 @@
       </c>
       <c r="D356" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E356" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F356" s="2" t="inlineStr"/>
-      <c r="G356" s="2" t="inlineStr"/>
-      <c r="H356" s="2" t="inlineStr"/>
-      <c r="I356" s="2" t="inlineStr"/>
-      <c r="J356" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F356" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G356" s="2" t="inlineStr">
+        <is>
+          <t>B08-G005</t>
+        </is>
+      </c>
+      <c r="H356" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I356" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J356" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K356" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L356" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -21731,27 +21831,47 @@
       </c>
       <c r="D357" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E357" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F357" s="2" t="inlineStr"/>
-      <c r="G357" s="2" t="inlineStr"/>
-      <c r="H357" s="2" t="inlineStr"/>
-      <c r="I357" s="2" t="inlineStr"/>
-      <c r="J357" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F357" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G357" s="2" t="inlineStr">
+        <is>
+          <t>B08-G006</t>
+        </is>
+      </c>
+      <c r="H357" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I357" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J357" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K357" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L357" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -21771,27 +21891,47 @@
       </c>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E358" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F358" s="2" t="inlineStr"/>
-      <c r="G358" s="2" t="inlineStr"/>
-      <c r="H358" s="2" t="inlineStr"/>
-      <c r="I358" s="2" t="inlineStr"/>
-      <c r="J358" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F358" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G358" s="2" t="inlineStr">
+        <is>
+          <t>B08-G007</t>
+        </is>
+      </c>
+      <c r="H358" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I358" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J358" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K358" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L358" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -21811,27 +21951,47 @@
       </c>
       <c r="D359" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E359" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F359" s="2" t="inlineStr"/>
-      <c r="G359" s="2" t="inlineStr"/>
-      <c r="H359" s="2" t="inlineStr"/>
-      <c r="I359" s="2" t="inlineStr"/>
-      <c r="J359" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F359" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G359" s="2" t="inlineStr">
+        <is>
+          <t>B08-G008</t>
+        </is>
+      </c>
+      <c r="H359" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I359" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J359" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K359" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L359" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -21851,27 +22011,47 @@
       </c>
       <c r="D360" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E360" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F360" s="2" t="inlineStr"/>
-      <c r="G360" s="2" t="inlineStr"/>
-      <c r="H360" s="2" t="inlineStr"/>
-      <c r="I360" s="2" t="inlineStr"/>
-      <c r="J360" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F360" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G360" s="2" t="inlineStr">
+        <is>
+          <t>B08-G009; B08-G010</t>
+        </is>
+      </c>
+      <c r="H360" s="2" t="inlineStr">
+        <is>
+          <t>multiple_single_page_instruments</t>
+        </is>
+      </c>
+      <c r="I360" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J360" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K360" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L360" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -21891,27 +22071,47 @@
       </c>
       <c r="D361" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E361" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F361" s="2" t="inlineStr"/>
-      <c r="G361" s="2" t="inlineStr"/>
-      <c r="H361" s="2" t="inlineStr"/>
-      <c r="I361" s="2" t="inlineStr"/>
-      <c r="J361" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F361" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G361" s="2" t="inlineStr">
+        <is>
+          <t>B08-G011; B08-G012</t>
+        </is>
+      </c>
+      <c r="H361" s="2" t="inlineStr">
+        <is>
+          <t>multiple_single_page_instruments</t>
+        </is>
+      </c>
+      <c r="I361" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J361" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K361" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L361" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -21931,27 +22131,47 @@
       </c>
       <c r="D362" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E362" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F362" s="2" t="inlineStr"/>
-      <c r="G362" s="2" t="inlineStr"/>
-      <c r="H362" s="2" t="inlineStr"/>
-      <c r="I362" s="2" t="inlineStr"/>
-      <c r="J362" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F362" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G362" s="2" t="inlineStr">
+        <is>
+          <t>B08-G013</t>
+        </is>
+      </c>
+      <c r="H362" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I362" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J362" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K362" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L362" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -21971,27 +22191,47 @@
       </c>
       <c r="D363" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E363" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F363" s="2" t="inlineStr"/>
-      <c r="G363" s="2" t="inlineStr"/>
-      <c r="H363" s="2" t="inlineStr"/>
-      <c r="I363" s="2" t="inlineStr"/>
-      <c r="J363" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F363" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G363" s="2" t="inlineStr">
+        <is>
+          <t>B08-G014</t>
+        </is>
+      </c>
+      <c r="H363" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I363" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J363" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K363" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L363" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22011,27 +22251,47 @@
       </c>
       <c r="D364" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E364" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F364" s="2" t="inlineStr"/>
-      <c r="G364" s="2" t="inlineStr"/>
-      <c r="H364" s="2" t="inlineStr"/>
-      <c r="I364" s="2" t="inlineStr"/>
-      <c r="J364" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F364" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G364" s="2" t="inlineStr">
+        <is>
+          <t>B08-G015</t>
+        </is>
+      </c>
+      <c r="H364" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I364" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J364" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K364" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L364" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22051,27 +22311,47 @@
       </c>
       <c r="D365" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E365" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F365" s="2" t="inlineStr"/>
-      <c r="G365" s="2" t="inlineStr"/>
-      <c r="H365" s="2" t="inlineStr"/>
-      <c r="I365" s="2" t="inlineStr"/>
-      <c r="J365" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F365" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G365" s="2" t="inlineStr">
+        <is>
+          <t>B08-G016</t>
+        </is>
+      </c>
+      <c r="H365" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I365" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J365" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K365" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L365" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22091,27 +22371,47 @@
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E366" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F366" s="2" t="inlineStr"/>
-      <c r="G366" s="2" t="inlineStr"/>
-      <c r="H366" s="2" t="inlineStr"/>
-      <c r="I366" s="2" t="inlineStr"/>
-      <c r="J366" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F366" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G366" s="2" t="inlineStr">
+        <is>
+          <t>B08-G017</t>
+        </is>
+      </c>
+      <c r="H366" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I366" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J366" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K366" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L366" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22131,27 +22431,47 @@
       </c>
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E367" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F367" s="2" t="inlineStr"/>
-      <c r="G367" s="2" t="inlineStr"/>
-      <c r="H367" s="2" t="inlineStr"/>
-      <c r="I367" s="2" t="inlineStr"/>
-      <c r="J367" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F367" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G367" s="2" t="inlineStr">
+        <is>
+          <t>B08-G018</t>
+        </is>
+      </c>
+      <c r="H367" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I367" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J367" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K367" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L367" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22171,27 +22491,47 @@
       </c>
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E368" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F368" s="2" t="inlineStr"/>
-      <c r="G368" s="2" t="inlineStr"/>
-      <c r="H368" s="2" t="inlineStr"/>
-      <c r="I368" s="2" t="inlineStr"/>
-      <c r="J368" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F368" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G368" s="2" t="inlineStr">
+        <is>
+          <t>B08-G019</t>
+        </is>
+      </c>
+      <c r="H368" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I368" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J368" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K368" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L368" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22211,27 +22551,47 @@
       </c>
       <c r="D369" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E369" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F369" s="2" t="inlineStr"/>
-      <c r="G369" s="2" t="inlineStr"/>
-      <c r="H369" s="2" t="inlineStr"/>
-      <c r="I369" s="2" t="inlineStr"/>
-      <c r="J369" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F369" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G369" s="2" t="inlineStr">
+        <is>
+          <t>B08-G020</t>
+        </is>
+      </c>
+      <c r="H369" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I369" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J369" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K369" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L369" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22251,27 +22611,47 @@
       </c>
       <c r="D370" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E370" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F370" s="2" t="inlineStr"/>
-      <c r="G370" s="2" t="inlineStr"/>
-      <c r="H370" s="2" t="inlineStr"/>
-      <c r="I370" s="2" t="inlineStr"/>
-      <c r="J370" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F370" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G370" s="2" t="inlineStr">
+        <is>
+          <t>B08-G021; B08-G022</t>
+        </is>
+      </c>
+      <c r="H370" s="2" t="inlineStr">
+        <is>
+          <t>multiple_single_page_instruments</t>
+        </is>
+      </c>
+      <c r="I370" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J370" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K370" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L370" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22291,27 +22671,47 @@
       </c>
       <c r="D371" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E371" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F371" s="2" t="inlineStr"/>
-      <c r="G371" s="2" t="inlineStr"/>
-      <c r="H371" s="2" t="inlineStr"/>
-      <c r="I371" s="2" t="inlineStr"/>
-      <c r="J371" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F371" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G371" s="2" t="inlineStr">
+        <is>
+          <t>B08-G023</t>
+        </is>
+      </c>
+      <c r="H371" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I371" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J371" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K371" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L371" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22331,27 +22731,47 @@
       </c>
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E372" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F372" s="2" t="inlineStr"/>
-      <c r="G372" s="2" t="inlineStr"/>
-      <c r="H372" s="2" t="inlineStr"/>
-      <c r="I372" s="2" t="inlineStr"/>
-      <c r="J372" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F372" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G372" s="2" t="inlineStr">
+        <is>
+          <t>B08-G024</t>
+        </is>
+      </c>
+      <c r="H372" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I372" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J372" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K372" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L372" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22371,27 +22791,47 @@
       </c>
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E373" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F373" s="2" t="inlineStr"/>
-      <c r="G373" s="2" t="inlineStr"/>
-      <c r="H373" s="2" t="inlineStr"/>
-      <c r="I373" s="2" t="inlineStr"/>
-      <c r="J373" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F373" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G373" s="2" t="inlineStr">
+        <is>
+          <t>B08-G025</t>
+        </is>
+      </c>
+      <c r="H373" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I373" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J373" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K373" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L373" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22411,27 +22851,47 @@
       </c>
       <c r="D374" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E374" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F374" s="2" t="inlineStr"/>
-      <c r="G374" s="2" t="inlineStr"/>
-      <c r="H374" s="2" t="inlineStr"/>
-      <c r="I374" s="2" t="inlineStr"/>
-      <c r="J374" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F374" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G374" s="2" t="inlineStr">
+        <is>
+          <t>B08-G025</t>
+        </is>
+      </c>
+      <c r="H374" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I374" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J374" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K374" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L374" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22451,27 +22911,47 @@
       </c>
       <c r="D375" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E375" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F375" s="2" t="inlineStr"/>
-      <c r="G375" s="2" t="inlineStr"/>
-      <c r="H375" s="2" t="inlineStr"/>
-      <c r="I375" s="2" t="inlineStr"/>
-      <c r="J375" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F375" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G375" s="2" t="inlineStr">
+        <is>
+          <t>B08-G026</t>
+        </is>
+      </c>
+      <c r="H375" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I375" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J375" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K375" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L375" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22491,27 +22971,47 @@
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E376" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F376" s="2" t="inlineStr"/>
-      <c r="G376" s="2" t="inlineStr"/>
-      <c r="H376" s="2" t="inlineStr"/>
-      <c r="I376" s="2" t="inlineStr"/>
-      <c r="J376" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F376" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G376" s="2" t="inlineStr">
+        <is>
+          <t>B08-G027</t>
+        </is>
+      </c>
+      <c r="H376" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I376" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J376" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K376" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L376" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22531,27 +23031,47 @@
       </c>
       <c r="D377" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E377" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F377" s="2" t="inlineStr"/>
-      <c r="G377" s="2" t="inlineStr"/>
-      <c r="H377" s="2" t="inlineStr"/>
-      <c r="I377" s="2" t="inlineStr"/>
-      <c r="J377" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F377" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G377" s="2" t="inlineStr">
+        <is>
+          <t>B08-G028</t>
+        </is>
+      </c>
+      <c r="H377" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I377" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J377" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K377" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L377" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22571,27 +23091,47 @@
       </c>
       <c r="D378" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E378" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F378" s="2" t="inlineStr"/>
-      <c r="G378" s="2" t="inlineStr"/>
-      <c r="H378" s="2" t="inlineStr"/>
-      <c r="I378" s="2" t="inlineStr"/>
-      <c r="J378" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F378" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G378" s="2" t="inlineStr">
+        <is>
+          <t>B08-G029; B08-G030</t>
+        </is>
+      </c>
+      <c r="H378" s="2" t="inlineStr">
+        <is>
+          <t>multiple_single_page_instruments</t>
+        </is>
+      </c>
+      <c r="I378" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J378" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K378" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L378" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22611,27 +23151,47 @@
       </c>
       <c r="D379" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E379" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F379" s="2" t="inlineStr"/>
-      <c r="G379" s="2" t="inlineStr"/>
-      <c r="H379" s="2" t="inlineStr"/>
-      <c r="I379" s="2" t="inlineStr"/>
-      <c r="J379" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F379" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G379" s="2" t="inlineStr">
+        <is>
+          <t>B08-G031</t>
+        </is>
+      </c>
+      <c r="H379" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I379" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J379" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K379" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L379" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22651,27 +23211,47 @@
       </c>
       <c r="D380" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E380" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F380" s="2" t="inlineStr"/>
-      <c r="G380" s="2" t="inlineStr"/>
-      <c r="H380" s="2" t="inlineStr"/>
-      <c r="I380" s="2" t="inlineStr"/>
-      <c r="J380" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F380" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G380" s="2" t="inlineStr">
+        <is>
+          <t>B08-G032</t>
+        </is>
+      </c>
+      <c r="H380" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I380" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J380" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K380" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L380" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22691,27 +23271,47 @@
       </c>
       <c r="D381" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E381" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F381" s="2" t="inlineStr"/>
-      <c r="G381" s="2" t="inlineStr"/>
-      <c r="H381" s="2" t="inlineStr"/>
-      <c r="I381" s="2" t="inlineStr"/>
-      <c r="J381" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F381" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G381" s="2" t="inlineStr">
+        <is>
+          <t>B08-G033</t>
+        </is>
+      </c>
+      <c r="H381" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I381" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J381" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K381" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L381" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22731,27 +23331,47 @@
       </c>
       <c r="D382" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E382" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F382" s="2" t="inlineStr"/>
-      <c r="G382" s="2" t="inlineStr"/>
-      <c r="H382" s="2" t="inlineStr"/>
-      <c r="I382" s="2" t="inlineStr"/>
-      <c r="J382" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F382" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G382" s="2" t="inlineStr">
+        <is>
+          <t>B08-G034</t>
+        </is>
+      </c>
+      <c r="H382" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I382" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J382" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K382" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L382" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22771,27 +23391,47 @@
       </c>
       <c r="D383" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E383" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F383" s="2" t="inlineStr"/>
-      <c r="G383" s="2" t="inlineStr"/>
-      <c r="H383" s="2" t="inlineStr"/>
-      <c r="I383" s="2" t="inlineStr"/>
-      <c r="J383" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F383" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G383" s="2" t="inlineStr">
+        <is>
+          <t>B08-G035</t>
+        </is>
+      </c>
+      <c r="H383" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I383" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J383" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K383" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L383" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22811,27 +23451,47 @@
       </c>
       <c r="D384" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E384" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F384" s="2" t="inlineStr"/>
-      <c r="G384" s="2" t="inlineStr"/>
-      <c r="H384" s="2" t="inlineStr"/>
-      <c r="I384" s="2" t="inlineStr"/>
-      <c r="J384" s="2" t="inlineStr"/>
+          <t>duplicate</t>
+        </is>
+      </c>
+      <c r="F384" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G384" s="2" t="inlineStr">
+        <is>
+          <t>B08-G036</t>
+        </is>
+      </c>
+      <c r="H384" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I384" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J384" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K384" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>duplicate_linked</t>
         </is>
       </c>
       <c r="L384" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22851,27 +23511,47 @@
       </c>
       <c r="D385" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E385" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F385" s="2" t="inlineStr"/>
-      <c r="G385" s="2" t="inlineStr"/>
-      <c r="H385" s="2" t="inlineStr"/>
-      <c r="I385" s="2" t="inlineStr"/>
-      <c r="J385" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F385" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G385" s="2" t="inlineStr">
+        <is>
+          <t>B08-G037</t>
+        </is>
+      </c>
+      <c r="H385" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I385" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J385" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K385" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L385" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22891,27 +23571,47 @@
       </c>
       <c r="D386" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E386" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F386" s="2" t="inlineStr"/>
-      <c r="G386" s="2" t="inlineStr"/>
-      <c r="H386" s="2" t="inlineStr"/>
-      <c r="I386" s="2" t="inlineStr"/>
-      <c r="J386" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F386" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G386" s="2" t="inlineStr">
+        <is>
+          <t>B08-G038</t>
+        </is>
+      </c>
+      <c r="H386" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I386" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J386" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K386" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L386" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22931,27 +23631,47 @@
       </c>
       <c r="D387" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E387" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F387" s="2" t="inlineStr"/>
-      <c r="G387" s="2" t="inlineStr"/>
-      <c r="H387" s="2" t="inlineStr"/>
-      <c r="I387" s="2" t="inlineStr"/>
-      <c r="J387" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F387" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G387" s="2" t="inlineStr">
+        <is>
+          <t>B08-G039</t>
+        </is>
+      </c>
+      <c r="H387" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I387" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J387" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K387" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L387" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -22971,27 +23691,47 @@
       </c>
       <c r="D388" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E388" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F388" s="2" t="inlineStr"/>
-      <c r="G388" s="2" t="inlineStr"/>
-      <c r="H388" s="2" t="inlineStr"/>
-      <c r="I388" s="2" t="inlineStr"/>
-      <c r="J388" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F388" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G388" s="2" t="inlineStr">
+        <is>
+          <t>B08-G040</t>
+        </is>
+      </c>
+      <c r="H388" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I388" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J388" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K388" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L388" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -23011,27 +23751,47 @@
       </c>
       <c r="D389" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E389" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F389" s="2" t="inlineStr"/>
-      <c r="G389" s="2" t="inlineStr"/>
-      <c r="H389" s="2" t="inlineStr"/>
-      <c r="I389" s="2" t="inlineStr"/>
-      <c r="J389" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F389" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G389" s="2" t="inlineStr">
+        <is>
+          <t>B08-G040</t>
+        </is>
+      </c>
+      <c r="H389" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I389" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J389" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K389" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L389" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -23051,27 +23811,47 @@
       </c>
       <c r="D390" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E390" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F390" s="2" t="inlineStr"/>
-      <c r="G390" s="2" t="inlineStr"/>
-      <c r="H390" s="2" t="inlineStr"/>
-      <c r="I390" s="2" t="inlineStr"/>
-      <c r="J390" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F390" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G390" s="2" t="inlineStr">
+        <is>
+          <t>B08-G041</t>
+        </is>
+      </c>
+      <c r="H390" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I390" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J390" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K390" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L390" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -23091,27 +23871,47 @@
       </c>
       <c r="D391" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E391" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F391" s="2" t="inlineStr"/>
-      <c r="G391" s="2" t="inlineStr"/>
-      <c r="H391" s="2" t="inlineStr"/>
-      <c r="I391" s="2" t="inlineStr"/>
-      <c r="J391" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F391" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G391" s="2" t="inlineStr">
+        <is>
+          <t>B08-G041</t>
+        </is>
+      </c>
+      <c r="H391" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I391" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J391" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K391" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L391" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -23131,27 +23931,47 @@
       </c>
       <c r="D392" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E392" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F392" s="2" t="inlineStr"/>
-      <c r="G392" s="2" t="inlineStr"/>
-      <c r="H392" s="2" t="inlineStr"/>
-      <c r="I392" s="2" t="inlineStr"/>
-      <c r="J392" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F392" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G392" s="2" t="inlineStr">
+        <is>
+          <t>B08-G042</t>
+        </is>
+      </c>
+      <c r="H392" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I392" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J392" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K392" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L392" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -23171,27 +23991,47 @@
       </c>
       <c r="D393" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E393" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F393" s="2" t="inlineStr"/>
-      <c r="G393" s="2" t="inlineStr"/>
-      <c r="H393" s="2" t="inlineStr"/>
-      <c r="I393" s="2" t="inlineStr"/>
-      <c r="J393" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F393" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G393" s="2" t="inlineStr">
+        <is>
+          <t>B08-G042</t>
+        </is>
+      </c>
+      <c r="H393" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I393" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J393" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K393" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L393" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -23211,27 +24051,47 @@
       </c>
       <c r="D394" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E394" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F394" s="2" t="inlineStr"/>
-      <c r="G394" s="2" t="inlineStr"/>
-      <c r="H394" s="2" t="inlineStr"/>
-      <c r="I394" s="2" t="inlineStr"/>
-      <c r="J394" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F394" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G394" s="2" t="inlineStr">
+        <is>
+          <t>B08-G043</t>
+        </is>
+      </c>
+      <c r="H394" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I394" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J394" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K394" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L394" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -23251,27 +24111,47 @@
       </c>
       <c r="D395" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E395" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F395" s="2" t="inlineStr"/>
-      <c r="G395" s="2" t="inlineStr"/>
-      <c r="H395" s="2" t="inlineStr"/>
-      <c r="I395" s="2" t="inlineStr"/>
-      <c r="J395" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F395" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G395" s="2" t="inlineStr">
+        <is>
+          <t>B08-G043</t>
+        </is>
+      </c>
+      <c r="H395" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I395" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J395" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K395" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L395" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -23291,27 +24171,47 @@
       </c>
       <c r="D396" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E396" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F396" s="2" t="inlineStr"/>
-      <c r="G396" s="2" t="inlineStr"/>
-      <c r="H396" s="2" t="inlineStr"/>
-      <c r="I396" s="2" t="inlineStr"/>
-      <c r="J396" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F396" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G396" s="2" t="inlineStr">
+        <is>
+          <t>B08-G044</t>
+        </is>
+      </c>
+      <c r="H396" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I396" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J396" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K396" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L396" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -23331,27 +24231,47 @@
       </c>
       <c r="D397" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E397" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F397" s="2" t="inlineStr"/>
-      <c r="G397" s="2" t="inlineStr"/>
-      <c r="H397" s="2" t="inlineStr"/>
-      <c r="I397" s="2" t="inlineStr"/>
-      <c r="J397" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F397" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G397" s="2" t="inlineStr">
+        <is>
+          <t>B08-G044</t>
+        </is>
+      </c>
+      <c r="H397" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I397" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J397" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K397" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L397" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -23371,27 +24291,47 @@
       </c>
       <c r="D398" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E398" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F398" s="2" t="inlineStr"/>
-      <c r="G398" s="2" t="inlineStr"/>
-      <c r="H398" s="2" t="inlineStr"/>
-      <c r="I398" s="2" t="inlineStr"/>
-      <c r="J398" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F398" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G398" s="2" t="inlineStr">
+        <is>
+          <t>B08-G045</t>
+        </is>
+      </c>
+      <c r="H398" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I398" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J398" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K398" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L398" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -23411,27 +24351,47 @@
       </c>
       <c r="D399" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E399" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F399" s="2" t="inlineStr"/>
-      <c r="G399" s="2" t="inlineStr"/>
-      <c r="H399" s="2" t="inlineStr"/>
-      <c r="I399" s="2" t="inlineStr"/>
-      <c r="J399" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F399" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G399" s="2" t="inlineStr">
+        <is>
+          <t>B08-G046</t>
+        </is>
+      </c>
+      <c r="H399" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I399" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J399" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K399" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L399" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -23451,27 +24411,47 @@
       </c>
       <c r="D400" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E400" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F400" s="2" t="inlineStr"/>
-      <c r="G400" s="2" t="inlineStr"/>
-      <c r="H400" s="2" t="inlineStr"/>
-      <c r="I400" s="2" t="inlineStr"/>
-      <c r="J400" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F400" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G400" s="2" t="inlineStr">
+        <is>
+          <t>B08-G036</t>
+        </is>
+      </c>
+      <c r="H400" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I400" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J400" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K400" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L400" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -23491,27 +24471,47 @@
       </c>
       <c r="D401" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E401" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F401" s="2" t="inlineStr"/>
-      <c r="G401" s="2" t="inlineStr"/>
-      <c r="H401" s="2" t="inlineStr"/>
-      <c r="I401" s="2" t="inlineStr"/>
-      <c r="J401" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F401" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G401" s="2" t="inlineStr">
+        <is>
+          <t>B08-G036</t>
+        </is>
+      </c>
+      <c r="H401" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I401" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J401" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K401" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L401" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR was used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Section 32 batch 09 checkpoint
Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
+++ b/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
@@ -24531,27 +24531,47 @@
       </c>
       <c r="D402" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E402" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F402" s="2" t="inlineStr"/>
-      <c r="G402" s="2" t="inlineStr"/>
-      <c r="H402" s="2" t="inlineStr"/>
-      <c r="I402" s="2" t="inlineStr"/>
-      <c r="J402" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F402" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G402" s="2" t="inlineStr">
+        <is>
+          <t>B09-G001</t>
+        </is>
+      </c>
+      <c r="H402" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I402" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J402" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K402" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L402" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -24571,27 +24591,47 @@
       </c>
       <c r="D403" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E403" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F403" s="2" t="inlineStr"/>
-      <c r="G403" s="2" t="inlineStr"/>
-      <c r="H403" s="2" t="inlineStr"/>
-      <c r="I403" s="2" t="inlineStr"/>
-      <c r="J403" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F403" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G403" s="2" t="inlineStr">
+        <is>
+          <t>B09-G002</t>
+        </is>
+      </c>
+      <c r="H403" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I403" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J403" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K403" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L403" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -24611,27 +24651,47 @@
       </c>
       <c r="D404" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E404" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F404" s="2" t="inlineStr"/>
-      <c r="G404" s="2" t="inlineStr"/>
-      <c r="H404" s="2" t="inlineStr"/>
-      <c r="I404" s="2" t="inlineStr"/>
-      <c r="J404" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F404" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G404" s="2" t="inlineStr">
+        <is>
+          <t>B09-G002</t>
+        </is>
+      </c>
+      <c r="H404" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I404" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J404" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K404" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L404" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -24651,27 +24711,47 @@
       </c>
       <c r="D405" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E405" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F405" s="2" t="inlineStr"/>
-      <c r="G405" s="2" t="inlineStr"/>
-      <c r="H405" s="2" t="inlineStr"/>
-      <c r="I405" s="2" t="inlineStr"/>
-      <c r="J405" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F405" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G405" s="2" t="inlineStr">
+        <is>
+          <t>B09-G003</t>
+        </is>
+      </c>
+      <c r="H405" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I405" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J405" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K405" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L405" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -24691,27 +24771,47 @@
       </c>
       <c r="D406" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E406" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F406" s="2" t="inlineStr"/>
-      <c r="G406" s="2" t="inlineStr"/>
-      <c r="H406" s="2" t="inlineStr"/>
-      <c r="I406" s="2" t="inlineStr"/>
-      <c r="J406" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F406" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G406" s="2" t="inlineStr">
+        <is>
+          <t>B09-G004</t>
+        </is>
+      </c>
+      <c r="H406" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I406" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J406" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K406" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L406" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -24731,27 +24831,47 @@
       </c>
       <c r="D407" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E407" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F407" s="2" t="inlineStr"/>
-      <c r="G407" s="2" t="inlineStr"/>
-      <c r="H407" s="2" t="inlineStr"/>
-      <c r="I407" s="2" t="inlineStr"/>
-      <c r="J407" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F407" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G407" s="2" t="inlineStr">
+        <is>
+          <t>B09-G004</t>
+        </is>
+      </c>
+      <c r="H407" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I407" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J407" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K407" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L407" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -24771,27 +24891,47 @@
       </c>
       <c r="D408" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E408" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F408" s="2" t="inlineStr"/>
-      <c r="G408" s="2" t="inlineStr"/>
-      <c r="H408" s="2" t="inlineStr"/>
-      <c r="I408" s="2" t="inlineStr"/>
-      <c r="J408" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F408" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G408" s="2" t="inlineStr">
+        <is>
+          <t>B09-G005</t>
+        </is>
+      </c>
+      <c r="H408" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I408" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J408" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K408" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L408" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -24811,27 +24951,47 @@
       </c>
       <c r="D409" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E409" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F409" s="2" t="inlineStr"/>
-      <c r="G409" s="2" t="inlineStr"/>
-      <c r="H409" s="2" t="inlineStr"/>
-      <c r="I409" s="2" t="inlineStr"/>
-      <c r="J409" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F409" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G409" s="2" t="inlineStr">
+        <is>
+          <t>B09-G006</t>
+        </is>
+      </c>
+      <c r="H409" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I409" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J409" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K409" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L409" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -24851,27 +25011,47 @@
       </c>
       <c r="D410" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E410" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F410" s="2" t="inlineStr"/>
-      <c r="G410" s="2" t="inlineStr"/>
-      <c r="H410" s="2" t="inlineStr"/>
-      <c r="I410" s="2" t="inlineStr"/>
-      <c r="J410" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F410" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G410" s="2" t="inlineStr">
+        <is>
+          <t>B09-G006</t>
+        </is>
+      </c>
+      <c r="H410" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I410" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J410" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K410" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L410" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -24891,27 +25071,47 @@
       </c>
       <c r="D411" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E411" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F411" s="2" t="inlineStr"/>
-      <c r="G411" s="2" t="inlineStr"/>
-      <c r="H411" s="2" t="inlineStr"/>
-      <c r="I411" s="2" t="inlineStr"/>
-      <c r="J411" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F411" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G411" s="2" t="inlineStr">
+        <is>
+          <t>B09-G007</t>
+        </is>
+      </c>
+      <c r="H411" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I411" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J411" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K411" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L411" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -24931,27 +25131,47 @@
       </c>
       <c r="D412" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E412" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F412" s="2" t="inlineStr"/>
-      <c r="G412" s="2" t="inlineStr"/>
-      <c r="H412" s="2" t="inlineStr"/>
-      <c r="I412" s="2" t="inlineStr"/>
-      <c r="J412" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F412" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G412" s="2" t="inlineStr">
+        <is>
+          <t>B09-G007</t>
+        </is>
+      </c>
+      <c r="H412" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I412" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J412" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K412" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L412" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -24971,27 +25191,47 @@
       </c>
       <c r="D413" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E413" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F413" s="2" t="inlineStr"/>
-      <c r="G413" s="2" t="inlineStr"/>
-      <c r="H413" s="2" t="inlineStr"/>
-      <c r="I413" s="2" t="inlineStr"/>
-      <c r="J413" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F413" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G413" s="2" t="inlineStr">
+        <is>
+          <t>B09-G008</t>
+        </is>
+      </c>
+      <c r="H413" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I413" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J413" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K413" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L413" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25011,27 +25251,47 @@
       </c>
       <c r="D414" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E414" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F414" s="2" t="inlineStr"/>
-      <c r="G414" s="2" t="inlineStr"/>
-      <c r="H414" s="2" t="inlineStr"/>
-      <c r="I414" s="2" t="inlineStr"/>
-      <c r="J414" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F414" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G414" s="2" t="inlineStr">
+        <is>
+          <t>B09-G008</t>
+        </is>
+      </c>
+      <c r="H414" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I414" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J414" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K414" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L414" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25051,27 +25311,47 @@
       </c>
       <c r="D415" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E415" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F415" s="2" t="inlineStr"/>
-      <c r="G415" s="2" t="inlineStr"/>
-      <c r="H415" s="2" t="inlineStr"/>
-      <c r="I415" s="2" t="inlineStr"/>
-      <c r="J415" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F415" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G415" s="2" t="inlineStr">
+        <is>
+          <t>B09-G009</t>
+        </is>
+      </c>
+      <c r="H415" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I415" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J415" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K415" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L415" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25091,27 +25371,47 @@
       </c>
       <c r="D416" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E416" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F416" s="2" t="inlineStr"/>
-      <c r="G416" s="2" t="inlineStr"/>
-      <c r="H416" s="2" t="inlineStr"/>
-      <c r="I416" s="2" t="inlineStr"/>
-      <c r="J416" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F416" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G416" s="2" t="inlineStr">
+        <is>
+          <t>B09-G010</t>
+        </is>
+      </c>
+      <c r="H416" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I416" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J416" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K416" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L416" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25131,27 +25431,47 @@
       </c>
       <c r="D417" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E417" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F417" s="2" t="inlineStr"/>
-      <c r="G417" s="2" t="inlineStr"/>
-      <c r="H417" s="2" t="inlineStr"/>
-      <c r="I417" s="2" t="inlineStr"/>
-      <c r="J417" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F417" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G417" s="2" t="inlineStr">
+        <is>
+          <t>B09-G011</t>
+        </is>
+      </c>
+      <c r="H417" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I417" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J417" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K417" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L417" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25171,27 +25491,47 @@
       </c>
       <c r="D418" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E418" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F418" s="2" t="inlineStr"/>
-      <c r="G418" s="2" t="inlineStr"/>
-      <c r="H418" s="2" t="inlineStr"/>
-      <c r="I418" s="2" t="inlineStr"/>
-      <c r="J418" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F418" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G418" s="2" t="inlineStr">
+        <is>
+          <t>B09-G012</t>
+        </is>
+      </c>
+      <c r="H418" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I418" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J418" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K418" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L418" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25211,27 +25551,47 @@
       </c>
       <c r="D419" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E419" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F419" s="2" t="inlineStr"/>
-      <c r="G419" s="2" t="inlineStr"/>
-      <c r="H419" s="2" t="inlineStr"/>
-      <c r="I419" s="2" t="inlineStr"/>
-      <c r="J419" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F419" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G419" s="2" t="inlineStr">
+        <is>
+          <t>B09-G013</t>
+        </is>
+      </c>
+      <c r="H419" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I419" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J419" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K419" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L419" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25251,27 +25611,47 @@
       </c>
       <c r="D420" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E420" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F420" s="2" t="inlineStr"/>
-      <c r="G420" s="2" t="inlineStr"/>
-      <c r="H420" s="2" t="inlineStr"/>
-      <c r="I420" s="2" t="inlineStr"/>
-      <c r="J420" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F420" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G420" s="2" t="inlineStr">
+        <is>
+          <t>B09-G014</t>
+        </is>
+      </c>
+      <c r="H420" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I420" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J420" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K420" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L420" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25291,27 +25671,47 @@
       </c>
       <c r="D421" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E421" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F421" s="2" t="inlineStr"/>
-      <c r="G421" s="2" t="inlineStr"/>
-      <c r="H421" s="2" t="inlineStr"/>
-      <c r="I421" s="2" t="inlineStr"/>
-      <c r="J421" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F421" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G421" s="2" t="inlineStr">
+        <is>
+          <t>B09-G015</t>
+        </is>
+      </c>
+      <c r="H421" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I421" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J421" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K421" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L421" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25331,27 +25731,47 @@
       </c>
       <c r="D422" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E422" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F422" s="2" t="inlineStr"/>
-      <c r="G422" s="2" t="inlineStr"/>
-      <c r="H422" s="2" t="inlineStr"/>
-      <c r="I422" s="2" t="inlineStr"/>
-      <c r="J422" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F422" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G422" s="2" t="inlineStr">
+        <is>
+          <t>B09-G016</t>
+        </is>
+      </c>
+      <c r="H422" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I422" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J422" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K422" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L422" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25371,27 +25791,47 @@
       </c>
       <c r="D423" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E423" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F423" s="2" t="inlineStr"/>
-      <c r="G423" s="2" t="inlineStr"/>
-      <c r="H423" s="2" t="inlineStr"/>
-      <c r="I423" s="2" t="inlineStr"/>
-      <c r="J423" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F423" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G423" s="2" t="inlineStr">
+        <is>
+          <t>B09-G017</t>
+        </is>
+      </c>
+      <c r="H423" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I423" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J423" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K423" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L423" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25411,27 +25851,47 @@
       </c>
       <c r="D424" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E424" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F424" s="2" t="inlineStr"/>
-      <c r="G424" s="2" t="inlineStr"/>
-      <c r="H424" s="2" t="inlineStr"/>
-      <c r="I424" s="2" t="inlineStr"/>
-      <c r="J424" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F424" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G424" s="2" t="inlineStr">
+        <is>
+          <t>B09-G018</t>
+        </is>
+      </c>
+      <c r="H424" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I424" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J424" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K424" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L424" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25451,27 +25911,47 @@
       </c>
       <c r="D425" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E425" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F425" s="2" t="inlineStr"/>
-      <c r="G425" s="2" t="inlineStr"/>
-      <c r="H425" s="2" t="inlineStr"/>
-      <c r="I425" s="2" t="inlineStr"/>
-      <c r="J425" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F425" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G425" s="2" t="inlineStr">
+        <is>
+          <t>B09-G019</t>
+        </is>
+      </c>
+      <c r="H425" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I425" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J425" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K425" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L425" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25491,27 +25971,47 @@
       </c>
       <c r="D426" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E426" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F426" s="2" t="inlineStr"/>
-      <c r="G426" s="2" t="inlineStr"/>
-      <c r="H426" s="2" t="inlineStr"/>
-      <c r="I426" s="2" t="inlineStr"/>
-      <c r="J426" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F426" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G426" s="2" t="inlineStr">
+        <is>
+          <t>B09-G019</t>
+        </is>
+      </c>
+      <c r="H426" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I426" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J426" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K426" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L426" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25531,27 +26031,47 @@
       </c>
       <c r="D427" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E427" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F427" s="2" t="inlineStr"/>
-      <c r="G427" s="2" t="inlineStr"/>
-      <c r="H427" s="2" t="inlineStr"/>
-      <c r="I427" s="2" t="inlineStr"/>
-      <c r="J427" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F427" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G427" s="2" t="inlineStr">
+        <is>
+          <t>B09-G020</t>
+        </is>
+      </c>
+      <c r="H427" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I427" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J427" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K427" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L427" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25571,27 +26091,47 @@
       </c>
       <c r="D428" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E428" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F428" s="2" t="inlineStr"/>
-      <c r="G428" s="2" t="inlineStr"/>
-      <c r="H428" s="2" t="inlineStr"/>
-      <c r="I428" s="2" t="inlineStr"/>
-      <c r="J428" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F428" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G428" s="2" t="inlineStr">
+        <is>
+          <t>B09-G020</t>
+        </is>
+      </c>
+      <c r="H428" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I428" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J428" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K428" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L428" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25611,27 +26151,47 @@
       </c>
       <c r="D429" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E429" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F429" s="2" t="inlineStr"/>
-      <c r="G429" s="2" t="inlineStr"/>
-      <c r="H429" s="2" t="inlineStr"/>
-      <c r="I429" s="2" t="inlineStr"/>
-      <c r="J429" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F429" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G429" s="2" t="inlineStr">
+        <is>
+          <t>B09-G021</t>
+        </is>
+      </c>
+      <c r="H429" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I429" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J429" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K429" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L429" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25651,27 +26211,47 @@
       </c>
       <c r="D430" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E430" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F430" s="2" t="inlineStr"/>
-      <c r="G430" s="2" t="inlineStr"/>
-      <c r="H430" s="2" t="inlineStr"/>
-      <c r="I430" s="2" t="inlineStr"/>
-      <c r="J430" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F430" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G430" s="2" t="inlineStr">
+        <is>
+          <t>B09-G021</t>
+        </is>
+      </c>
+      <c r="H430" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I430" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J430" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K430" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L430" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25691,27 +26271,47 @@
       </c>
       <c r="D431" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E431" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F431" s="2" t="inlineStr"/>
-      <c r="G431" s="2" t="inlineStr"/>
-      <c r="H431" s="2" t="inlineStr"/>
-      <c r="I431" s="2" t="inlineStr"/>
-      <c r="J431" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F431" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G431" s="2" t="inlineStr">
+        <is>
+          <t>B09-G022</t>
+        </is>
+      </c>
+      <c r="H431" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I431" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J431" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K431" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L431" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25731,27 +26331,47 @@
       </c>
       <c r="D432" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E432" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F432" s="2" t="inlineStr"/>
-      <c r="G432" s="2" t="inlineStr"/>
-      <c r="H432" s="2" t="inlineStr"/>
-      <c r="I432" s="2" t="inlineStr"/>
-      <c r="J432" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F432" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G432" s="2" t="inlineStr">
+        <is>
+          <t>B09-G022</t>
+        </is>
+      </c>
+      <c r="H432" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I432" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J432" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K432" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L432" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25771,27 +26391,47 @@
       </c>
       <c r="D433" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E433" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F433" s="2" t="inlineStr"/>
-      <c r="G433" s="2" t="inlineStr"/>
-      <c r="H433" s="2" t="inlineStr"/>
-      <c r="I433" s="2" t="inlineStr"/>
-      <c r="J433" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F433" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G433" s="2" t="inlineStr">
+        <is>
+          <t>B09-G023</t>
+        </is>
+      </c>
+      <c r="H433" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I433" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J433" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K433" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L433" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25811,27 +26451,47 @@
       </c>
       <c r="D434" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E434" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F434" s="2" t="inlineStr"/>
-      <c r="G434" s="2" t="inlineStr"/>
-      <c r="H434" s="2" t="inlineStr"/>
-      <c r="I434" s="2" t="inlineStr"/>
-      <c r="J434" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F434" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G434" s="2" t="inlineStr">
+        <is>
+          <t>B09-G023</t>
+        </is>
+      </c>
+      <c r="H434" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I434" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J434" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K434" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L434" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25851,27 +26511,47 @@
       </c>
       <c r="D435" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E435" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F435" s="2" t="inlineStr"/>
-      <c r="G435" s="2" t="inlineStr"/>
-      <c r="H435" s="2" t="inlineStr"/>
-      <c r="I435" s="2" t="inlineStr"/>
-      <c r="J435" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F435" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G435" s="2" t="inlineStr">
+        <is>
+          <t>B09-G024</t>
+        </is>
+      </c>
+      <c r="H435" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I435" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J435" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K435" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L435" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25891,27 +26571,47 @@
       </c>
       <c r="D436" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E436" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F436" s="2" t="inlineStr"/>
-      <c r="G436" s="2" t="inlineStr"/>
-      <c r="H436" s="2" t="inlineStr"/>
-      <c r="I436" s="2" t="inlineStr"/>
-      <c r="J436" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F436" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G436" s="2" t="inlineStr">
+        <is>
+          <t>B09-G024</t>
+        </is>
+      </c>
+      <c r="H436" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I436" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J436" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K436" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L436" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25931,27 +26631,47 @@
       </c>
       <c r="D437" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E437" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F437" s="2" t="inlineStr"/>
-      <c r="G437" s="2" t="inlineStr"/>
-      <c r="H437" s="2" t="inlineStr"/>
-      <c r="I437" s="2" t="inlineStr"/>
-      <c r="J437" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F437" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G437" s="2" t="inlineStr">
+        <is>
+          <t>B09-G025</t>
+        </is>
+      </c>
+      <c r="H437" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I437" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J437" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K437" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L437" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -25971,27 +26691,47 @@
       </c>
       <c r="D438" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E438" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F438" s="2" t="inlineStr"/>
-      <c r="G438" s="2" t="inlineStr"/>
-      <c r="H438" s="2" t="inlineStr"/>
-      <c r="I438" s="2" t="inlineStr"/>
-      <c r="J438" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F438" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G438" s="2" t="inlineStr">
+        <is>
+          <t>B09-G026</t>
+        </is>
+      </c>
+      <c r="H438" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I438" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J438" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K438" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L438" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -26011,27 +26751,47 @@
       </c>
       <c r="D439" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E439" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F439" s="2" t="inlineStr"/>
-      <c r="G439" s="2" t="inlineStr"/>
-      <c r="H439" s="2" t="inlineStr"/>
-      <c r="I439" s="2" t="inlineStr"/>
-      <c r="J439" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F439" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G439" s="2" t="inlineStr">
+        <is>
+          <t>B09-G027</t>
+        </is>
+      </c>
+      <c r="H439" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I439" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J439" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K439" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L439" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -26051,27 +26811,47 @@
       </c>
       <c r="D440" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E440" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F440" s="2" t="inlineStr"/>
-      <c r="G440" s="2" t="inlineStr"/>
-      <c r="H440" s="2" t="inlineStr"/>
-      <c r="I440" s="2" t="inlineStr"/>
-      <c r="J440" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F440" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G440" s="2" t="inlineStr">
+        <is>
+          <t>B09-G028</t>
+        </is>
+      </c>
+      <c r="H440" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I440" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J440" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K440" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L440" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -26091,27 +26871,47 @@
       </c>
       <c r="D441" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E441" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F441" s="2" t="inlineStr"/>
-      <c r="G441" s="2" t="inlineStr"/>
-      <c r="H441" s="2" t="inlineStr"/>
-      <c r="I441" s="2" t="inlineStr"/>
-      <c r="J441" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F441" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G441" s="2" t="inlineStr">
+        <is>
+          <t>B09-G029</t>
+        </is>
+      </c>
+      <c r="H441" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I441" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J441" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K441" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L441" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -26131,27 +26931,47 @@
       </c>
       <c r="D442" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E442" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F442" s="2" t="inlineStr"/>
-      <c r="G442" s="2" t="inlineStr"/>
-      <c r="H442" s="2" t="inlineStr"/>
-      <c r="I442" s="2" t="inlineStr"/>
-      <c r="J442" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F442" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G442" s="2" t="inlineStr">
+        <is>
+          <t>B09-G030</t>
+        </is>
+      </c>
+      <c r="H442" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I442" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J442" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K442" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L442" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -26171,27 +26991,47 @@
       </c>
       <c r="D443" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E443" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F443" s="2" t="inlineStr"/>
-      <c r="G443" s="2" t="inlineStr"/>
-      <c r="H443" s="2" t="inlineStr"/>
-      <c r="I443" s="2" t="inlineStr"/>
-      <c r="J443" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F443" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G443" s="2" t="inlineStr">
+        <is>
+          <t>B09-G031</t>
+        </is>
+      </c>
+      <c r="H443" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I443" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J443" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K443" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L443" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -26211,27 +27051,47 @@
       </c>
       <c r="D444" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E444" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F444" s="2" t="inlineStr"/>
-      <c r="G444" s="2" t="inlineStr"/>
-      <c r="H444" s="2" t="inlineStr"/>
-      <c r="I444" s="2" t="inlineStr"/>
-      <c r="J444" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F444" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G444" s="2" t="inlineStr">
+        <is>
+          <t>B09-G031</t>
+        </is>
+      </c>
+      <c r="H444" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I444" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J444" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K444" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L444" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -26251,27 +27111,47 @@
       </c>
       <c r="D445" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E445" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F445" s="2" t="inlineStr"/>
-      <c r="G445" s="2" t="inlineStr"/>
-      <c r="H445" s="2" t="inlineStr"/>
-      <c r="I445" s="2" t="inlineStr"/>
-      <c r="J445" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F445" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G445" s="2" t="inlineStr">
+        <is>
+          <t>B09-G032</t>
+        </is>
+      </c>
+      <c r="H445" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I445" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J445" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K445" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L445" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -26291,27 +27171,47 @@
       </c>
       <c r="D446" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E446" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F446" s="2" t="inlineStr"/>
-      <c r="G446" s="2" t="inlineStr"/>
-      <c r="H446" s="2" t="inlineStr"/>
-      <c r="I446" s="2" t="inlineStr"/>
-      <c r="J446" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F446" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G446" s="2" t="inlineStr">
+        <is>
+          <t>B09-G032</t>
+        </is>
+      </c>
+      <c r="H446" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I446" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J446" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K446" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L446" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -26331,27 +27231,47 @@
       </c>
       <c r="D447" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E447" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F447" s="2" t="inlineStr"/>
-      <c r="G447" s="2" t="inlineStr"/>
-      <c r="H447" s="2" t="inlineStr"/>
-      <c r="I447" s="2" t="inlineStr"/>
-      <c r="J447" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F447" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G447" s="2" t="inlineStr">
+        <is>
+          <t>B09-G033</t>
+        </is>
+      </c>
+      <c r="H447" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I447" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J447" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K447" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L447" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -26371,27 +27291,47 @@
       </c>
       <c r="D448" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E448" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F448" s="2" t="inlineStr"/>
-      <c r="G448" s="2" t="inlineStr"/>
-      <c r="H448" s="2" t="inlineStr"/>
-      <c r="I448" s="2" t="inlineStr"/>
-      <c r="J448" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F448" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G448" s="2" t="inlineStr">
+        <is>
+          <t>B09-G034</t>
+        </is>
+      </c>
+      <c r="H448" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I448" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J448" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K448" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L448" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -26411,27 +27351,47 @@
       </c>
       <c r="D449" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E449" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F449" s="2" t="inlineStr"/>
-      <c r="G449" s="2" t="inlineStr"/>
-      <c r="H449" s="2" t="inlineStr"/>
-      <c r="I449" s="2" t="inlineStr"/>
-      <c r="J449" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F449" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G449" s="2" t="inlineStr">
+        <is>
+          <t>B09-G035</t>
+        </is>
+      </c>
+      <c r="H449" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I449" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J449" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K449" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L449" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -26451,27 +27411,47 @@
       </c>
       <c r="D450" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E450" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F450" s="2" t="inlineStr"/>
-      <c r="G450" s="2" t="inlineStr"/>
-      <c r="H450" s="2" t="inlineStr"/>
-      <c r="I450" s="2" t="inlineStr"/>
-      <c r="J450" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F450" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G450" s="2" t="inlineStr">
+        <is>
+          <t>B09-G036</t>
+        </is>
+      </c>
+      <c r="H450" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I450" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J450" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K450" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L450" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>
@@ -26491,27 +27471,47 @@
       </c>
       <c r="D451" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E451" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F451" s="2" t="inlineStr"/>
-      <c r="G451" s="2" t="inlineStr"/>
-      <c r="H451" s="2" t="inlineStr"/>
-      <c r="I451" s="2" t="inlineStr"/>
-      <c r="J451" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F451" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G451" s="2" t="inlineStr">
+        <is>
+          <t>B09-G037</t>
+        </is>
+      </c>
+      <c r="H451" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I451" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J451" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K451" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L451" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Visually inspected directly at readable scale; OCR used only as an aid. Stamps, signatures, acknowledgments, marginal notes, schedules, and page continuity were checked.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Section 32 batch 10 and final workbook
Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
+++ b/artifacts/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_2026-07-15/SECTION32_IMAGES_0001_0500_GPT-5-6-SOL_IMAGE_INVENTORY.xlsx
@@ -27531,27 +27531,47 @@
       </c>
       <c r="D452" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E452" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F452" s="2" t="inlineStr"/>
-      <c r="G452" s="2" t="inlineStr"/>
-      <c r="H452" s="2" t="inlineStr"/>
-      <c r="I452" s="2" t="inlineStr"/>
-      <c r="J452" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F452" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G452" s="2" t="inlineStr">
+        <is>
+          <t>B10-G001</t>
+        </is>
+      </c>
+      <c r="H452" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I452" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J452" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K452" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L452" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Mineral deed; recording stamp, signatures, acknowledgment, and legal description inspected.</t>
         </is>
       </c>
     </row>
@@ -27571,27 +27591,47 @@
       </c>
       <c r="D453" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E453" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F453" s="2" t="inlineStr"/>
-      <c r="G453" s="2" t="inlineStr"/>
-      <c r="H453" s="2" t="inlineStr"/>
-      <c r="I453" s="2" t="inlineStr"/>
-      <c r="J453" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F453" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G453" s="2" t="inlineStr">
+        <is>
+          <t>B10-G002</t>
+        </is>
+      </c>
+      <c r="H453" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I453" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J453" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K453" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L453" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Multi-tract mineral deed; all visible calls and recording stamp inspected.</t>
         </is>
       </c>
     </row>
@@ -27611,27 +27651,47 @@
       </c>
       <c r="D454" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E454" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F454" s="2" t="inlineStr"/>
-      <c r="G454" s="2" t="inlineStr"/>
-      <c r="H454" s="2" t="inlineStr"/>
-      <c r="I454" s="2" t="inlineStr"/>
-      <c r="J454" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F454" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G454" s="2" t="inlineStr">
+        <is>
+          <t>B10-G003</t>
+        </is>
+      </c>
+      <c r="H454" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I454" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J454" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K454" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L454" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Mineral deed; handwritten correction, signatures, acknowledgment, stamps, and legal inspected.</t>
         </is>
       </c>
     </row>
@@ -27651,27 +27711,47 @@
       </c>
       <c r="D455" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E455" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F455" s="2" t="inlineStr"/>
-      <c r="G455" s="2" t="inlineStr"/>
-      <c r="H455" s="2" t="inlineStr"/>
-      <c r="I455" s="2" t="inlineStr"/>
-      <c r="J455" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F455" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G455" s="2" t="inlineStr">
+        <is>
+          <t>B10-G004</t>
+        </is>
+      </c>
+      <c r="H455" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I455" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J455" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K455" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L455" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Handwritten mineral deed; intent clause and acknowledgment inspected.</t>
         </is>
       </c>
     </row>
@@ -27691,27 +27771,47 @@
       </c>
       <c r="D456" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E456" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F456" s="2" t="inlineStr"/>
-      <c r="G456" s="2" t="inlineStr"/>
-      <c r="H456" s="2" t="inlineStr"/>
-      <c r="I456" s="2" t="inlineStr"/>
-      <c r="J456" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F456" s="2" t="inlineStr">
+        <is>
+          <t>fair</t>
+        </is>
+      </c>
+      <c r="G456" s="2" t="inlineStr">
+        <is>
+          <t>B10-G005</t>
+        </is>
+      </c>
+      <c r="H456" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I456" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J456" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K456" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted_with_assumption</t>
         </is>
       </c>
       <c r="L456" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Multi-tract mineral deed enlarged and cropped; Section 32 fraction read as 54/640ths.</t>
         </is>
       </c>
     </row>
@@ -27731,27 +27831,47 @@
       </c>
       <c r="D457" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E457" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F457" s="2" t="inlineStr"/>
-      <c r="G457" s="2" t="inlineStr"/>
-      <c r="H457" s="2" t="inlineStr"/>
-      <c r="I457" s="2" t="inlineStr"/>
-      <c r="J457" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F457" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G457" s="2" t="inlineStr">
+        <is>
+          <t>B10-G006</t>
+        </is>
+      </c>
+      <c r="H457" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I457" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J457" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K457" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L457" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Mineral deed; stamps, signatures, acknowledgment, and intent clause inspected.</t>
         </is>
       </c>
     </row>
@@ -27771,27 +27891,47 @@
       </c>
       <c r="D458" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E458" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F458" s="2" t="inlineStr"/>
-      <c r="G458" s="2" t="inlineStr"/>
-      <c r="H458" s="2" t="inlineStr"/>
-      <c r="I458" s="2" t="inlineStr"/>
-      <c r="J458" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F458" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G458" s="2" t="inlineStr">
+        <is>
+          <t>B10-G007</t>
+        </is>
+      </c>
+      <c r="H458" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I458" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J458" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K458" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L458" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Mineral deed; stamps, signatures, acknowledgment, and legal inspected.</t>
         </is>
       </c>
     </row>
@@ -27811,27 +27951,47 @@
       </c>
       <c r="D459" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E459" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F459" s="2" t="inlineStr"/>
-      <c r="G459" s="2" t="inlineStr"/>
-      <c r="H459" s="2" t="inlineStr"/>
-      <c r="I459" s="2" t="inlineStr"/>
-      <c r="J459" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F459" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G459" s="2" t="inlineStr">
+        <is>
+          <t>B10-G008</t>
+        </is>
+      </c>
+      <c r="H459" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I459" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J459" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K459" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L459" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>First page of multi-tract mineral deed; fractions and legal schedule inspected.</t>
         </is>
       </c>
     </row>
@@ -27851,27 +28011,47 @@
       </c>
       <c r="D460" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E460" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F460" s="2" t="inlineStr"/>
-      <c r="G460" s="2" t="inlineStr"/>
-      <c r="H460" s="2" t="inlineStr"/>
-      <c r="I460" s="2" t="inlineStr"/>
-      <c r="J460" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F460" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G460" s="2" t="inlineStr">
+        <is>
+          <t>B10-G008</t>
+        </is>
+      </c>
+      <c r="H460" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I460" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J460" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K460" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L460" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Acknowledgment and recording continuation of 0458.</t>
         </is>
       </c>
     </row>
@@ -27891,27 +28071,47 @@
       </c>
       <c r="D461" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E461" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F461" s="2" t="inlineStr"/>
-      <c r="G461" s="2" t="inlineStr"/>
-      <c r="H461" s="2" t="inlineStr"/>
-      <c r="I461" s="2" t="inlineStr"/>
-      <c r="J461" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F461" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G461" s="2" t="inlineStr">
+        <is>
+          <t>B10-G009</t>
+        </is>
+      </c>
+      <c r="H461" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I461" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J461" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K461" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L461" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Mineral deed; legal, execution, acknowledgment, and stamp inspected.</t>
         </is>
       </c>
     </row>
@@ -27931,27 +28131,47 @@
       </c>
       <c r="D462" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E462" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F462" s="2" t="inlineStr"/>
-      <c r="G462" s="2" t="inlineStr"/>
-      <c r="H462" s="2" t="inlineStr"/>
-      <c r="I462" s="2" t="inlineStr"/>
-      <c r="J462" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F462" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G462" s="2" t="inlineStr">
+        <is>
+          <t>B10-G010</t>
+        </is>
+      </c>
+      <c r="H462" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I462" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J462" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K462" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L462" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Mineral deed; legal, execution, acknowledgment, and stamp inspected.</t>
         </is>
       </c>
     </row>
@@ -27971,27 +28191,47 @@
       </c>
       <c r="D463" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E463" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F463" s="2" t="inlineStr"/>
-      <c r="G463" s="2" t="inlineStr"/>
-      <c r="H463" s="2" t="inlineStr"/>
-      <c r="I463" s="2" t="inlineStr"/>
-      <c r="J463" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F463" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G463" s="2" t="inlineStr">
+        <is>
+          <t>B10-G011</t>
+        </is>
+      </c>
+      <c r="H463" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I463" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J463" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K463" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L463" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Mineral deed; homestead statement, legal, and acknowledgment inspected.</t>
         </is>
       </c>
     </row>
@@ -28011,27 +28251,47 @@
       </c>
       <c r="D464" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E464" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F464" s="2" t="inlineStr"/>
-      <c r="G464" s="2" t="inlineStr"/>
-      <c r="H464" s="2" t="inlineStr"/>
-      <c r="I464" s="2" t="inlineStr"/>
-      <c r="J464" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F464" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G464" s="2" t="inlineStr">
+        <is>
+          <t>B10-G012</t>
+        </is>
+      </c>
+      <c r="H464" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I464" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J464" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K464" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L464" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Mineral deed; corporate grantee identity and acknowledgment inspected.</t>
         </is>
       </c>
     </row>
@@ -28051,27 +28311,47 @@
       </c>
       <c r="D465" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E465" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F465" s="2" t="inlineStr"/>
-      <c r="G465" s="2" t="inlineStr"/>
-      <c r="H465" s="2" t="inlineStr"/>
-      <c r="I465" s="2" t="inlineStr"/>
-      <c r="J465" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F465" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G465" s="2" t="inlineStr">
+        <is>
+          <t>B10-G013</t>
+        </is>
+      </c>
+      <c r="H465" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I465" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J465" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K465" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L465" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Designation of depository first page; lease reference, bank, execution, and marginal notes inspected.</t>
         </is>
       </c>
     </row>
@@ -28091,27 +28371,47 @@
       </c>
       <c r="D466" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E466" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F466" s="2" t="inlineStr"/>
-      <c r="G466" s="2" t="inlineStr"/>
-      <c r="H466" s="2" t="inlineStr"/>
-      <c r="I466" s="2" t="inlineStr"/>
-      <c r="J466" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F466" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G466" s="2" t="inlineStr">
+        <is>
+          <t>B10-G013</t>
+        </is>
+      </c>
+      <c r="H466" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I466" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J466" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K466" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L466" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Acknowledgment and return-address continuation of 0464; page rotated mentally for inspection.</t>
         </is>
       </c>
     </row>
@@ -28131,27 +28431,47 @@
       </c>
       <c r="D467" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E467" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F467" s="2" t="inlineStr"/>
-      <c r="G467" s="2" t="inlineStr"/>
-      <c r="H467" s="2" t="inlineStr"/>
-      <c r="I467" s="2" t="inlineStr"/>
-      <c r="J467" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F467" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G467" s="2" t="inlineStr">
+        <is>
+          <t>B10-G014</t>
+        </is>
+      </c>
+      <c r="H467" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I467" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J467" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K467" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L467" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Corporate mineral deed with multi-tract schedule; Section 32 call inspected.</t>
         </is>
       </c>
     </row>
@@ -28171,27 +28491,47 @@
       </c>
       <c r="D468" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E468" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F468" s="2" t="inlineStr"/>
-      <c r="G468" s="2" t="inlineStr"/>
-      <c r="H468" s="2" t="inlineStr"/>
-      <c r="I468" s="2" t="inlineStr"/>
-      <c r="J468" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F468" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G468" s="2" t="inlineStr">
+        <is>
+          <t>B10-G015</t>
+        </is>
+      </c>
+      <c r="H468" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I468" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J468" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K468" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L468" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Mineral deed; effective-date clause, homestead statement, and recording stamp inspected.</t>
         </is>
       </c>
     </row>
@@ -28211,27 +28551,47 @@
       </c>
       <c r="D469" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E469" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F469" s="2" t="inlineStr"/>
-      <c r="G469" s="2" t="inlineStr"/>
-      <c r="H469" s="2" t="inlineStr"/>
-      <c r="I469" s="2" t="inlineStr"/>
-      <c r="J469" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F469" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G469" s="2" t="inlineStr">
+        <is>
+          <t>B10-G016</t>
+        </is>
+      </c>
+      <c r="H469" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I469" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J469" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K469" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L469" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Separate mineral deed despite repeated form number; legal and stamp inspected.</t>
         </is>
       </c>
     </row>
@@ -28251,27 +28611,47 @@
       </c>
       <c r="D470" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E470" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F470" s="2" t="inlineStr"/>
-      <c r="G470" s="2" t="inlineStr"/>
-      <c r="H470" s="2" t="inlineStr"/>
-      <c r="I470" s="2" t="inlineStr"/>
-      <c r="J470" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F470" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G470" s="2" t="inlineStr">
+        <is>
+          <t>B10-G017</t>
+        </is>
+      </c>
+      <c r="H470" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I470" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J470" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K470" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L470" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Designation of depository first page; Maddoux lease and bank designation inspected.</t>
         </is>
       </c>
     </row>
@@ -28291,27 +28671,47 @@
       </c>
       <c r="D471" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E471" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F471" s="2" t="inlineStr"/>
-      <c r="G471" s="2" t="inlineStr"/>
-      <c r="H471" s="2" t="inlineStr"/>
-      <c r="I471" s="2" t="inlineStr"/>
-      <c r="J471" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F471" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G471" s="2" t="inlineStr">
+        <is>
+          <t>B10-G017</t>
+        </is>
+      </c>
+      <c r="H471" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I471" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J471" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K471" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L471" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Acknowledgment and recording continuation of 0469; sideways form inspected.</t>
         </is>
       </c>
     </row>
@@ -28331,27 +28731,47 @@
       </c>
       <c r="D472" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E472" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F472" s="2" t="inlineStr"/>
-      <c r="G472" s="2" t="inlineStr"/>
-      <c r="H472" s="2" t="inlineStr"/>
-      <c r="I472" s="2" t="inlineStr"/>
-      <c r="J472" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F472" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G472" s="2" t="inlineStr">
+        <is>
+          <t>B10-G018</t>
+        </is>
+      </c>
+      <c r="H472" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I472" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J472" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K472" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L472" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Designation of depository first page; Garrett lease and bank designation inspected.</t>
         </is>
       </c>
     </row>
@@ -28371,27 +28791,47 @@
       </c>
       <c r="D473" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E473" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F473" s="2" t="inlineStr"/>
-      <c r="G473" s="2" t="inlineStr"/>
-      <c r="H473" s="2" t="inlineStr"/>
-      <c r="I473" s="2" t="inlineStr"/>
-      <c r="J473" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F473" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G473" s="2" t="inlineStr">
+        <is>
+          <t>B10-G018</t>
+        </is>
+      </c>
+      <c r="H473" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I473" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J473" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K473" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L473" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Acknowledgment and recording continuation of 0471; sideways form inspected.</t>
         </is>
       </c>
     </row>
@@ -28411,27 +28851,47 @@
       </c>
       <c r="D474" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E474" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F474" s="2" t="inlineStr"/>
-      <c r="G474" s="2" t="inlineStr"/>
-      <c r="H474" s="2" t="inlineStr"/>
-      <c r="I474" s="2" t="inlineStr"/>
-      <c r="J474" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F474" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G474" s="2" t="inlineStr">
+        <is>
+          <t>B10-G019</t>
+        </is>
+      </c>
+      <c r="H474" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I474" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J474" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K474" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L474" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Assignment of oil and gas leases; fractional assignees, execution, and acknowledgment inspected.</t>
         </is>
       </c>
     </row>
@@ -28451,27 +28911,47 @@
       </c>
       <c r="D475" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E475" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F475" s="2" t="inlineStr"/>
-      <c r="G475" s="2" t="inlineStr"/>
-      <c r="H475" s="2" t="inlineStr"/>
-      <c r="I475" s="2" t="inlineStr"/>
-      <c r="J475" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F475" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G475" s="2" t="inlineStr">
+        <is>
+          <t>B10-G019</t>
+        </is>
+      </c>
+      <c r="H475" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I475" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J475" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K475" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L475" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Exhibit A page 1; lease numbers, lessors, record references, and descriptions inspected.</t>
         </is>
       </c>
     </row>
@@ -28491,27 +28971,47 @@
       </c>
       <c r="D476" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E476" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F476" s="2" t="inlineStr"/>
-      <c r="G476" s="2" t="inlineStr"/>
-      <c r="H476" s="2" t="inlineStr"/>
-      <c r="I476" s="2" t="inlineStr"/>
-      <c r="J476" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F476" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G476" s="2" t="inlineStr">
+        <is>
+          <t>B10-G019</t>
+        </is>
+      </c>
+      <c r="H476" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I476" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J476" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K476" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L476" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Exhibit A page 2; lease schedule inspected.</t>
         </is>
       </c>
     </row>
@@ -28531,27 +29031,47 @@
       </c>
       <c r="D477" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E477" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F477" s="2" t="inlineStr"/>
-      <c r="G477" s="2" t="inlineStr"/>
-      <c r="H477" s="2" t="inlineStr"/>
-      <c r="I477" s="2" t="inlineStr"/>
-      <c r="J477" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F477" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G477" s="2" t="inlineStr">
+        <is>
+          <t>B10-G019</t>
+        </is>
+      </c>
+      <c r="H477" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I477" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J477" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K477" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L477" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Exhibit A page 3 and recording stamp; final page of assignment inspected.</t>
         </is>
       </c>
     </row>
@@ -28571,27 +29091,47 @@
       </c>
       <c r="D478" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E478" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F478" s="2" t="inlineStr"/>
-      <c r="G478" s="2" t="inlineStr"/>
-      <c r="H478" s="2" t="inlineStr"/>
-      <c r="I478" s="2" t="inlineStr"/>
-      <c r="J478" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F478" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G478" s="2" t="inlineStr">
+        <is>
+          <t>B10-G020</t>
+        </is>
+      </c>
+      <c r="H478" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I478" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J478" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K478" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted_not_section_32</t>
         </is>
       </c>
       <c r="L478" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Lease ratification concerns Section 28 only; acquired-interest clause and acknowledgment inspected.</t>
         </is>
       </c>
     </row>
@@ -28611,27 +29151,47 @@
       </c>
       <c r="D479" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E479" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F479" s="2" t="inlineStr"/>
-      <c r="G479" s="2" t="inlineStr"/>
-      <c r="H479" s="2" t="inlineStr"/>
-      <c r="I479" s="2" t="inlineStr"/>
-      <c r="J479" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F479" s="2" t="inlineStr">
+        <is>
+          <t>fair-to-good</t>
+        </is>
+      </c>
+      <c r="G479" s="2" t="inlineStr">
+        <is>
+          <t>B10-G021</t>
+        </is>
+      </c>
+      <c r="H479" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I479" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J479" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K479" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L479" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Multi-tract mineral deed first page; Section 32 calls and joint-tenancy language inspected.</t>
         </is>
       </c>
     </row>
@@ -28651,27 +29211,47 @@
       </c>
       <c r="D480" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E480" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F480" s="2" t="inlineStr"/>
-      <c r="G480" s="2" t="inlineStr"/>
-      <c r="H480" s="2" t="inlineStr"/>
-      <c r="I480" s="2" t="inlineStr"/>
-      <c r="J480" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F480" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G480" s="2" t="inlineStr">
+        <is>
+          <t>B10-G021</t>
+        </is>
+      </c>
+      <c r="H480" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I480" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J480" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K480" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L480" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Execution and corporate acknowledgment continuation of 0478.</t>
         </is>
       </c>
     </row>
@@ -28691,27 +29271,47 @@
       </c>
       <c r="D481" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E481" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F481" s="2" t="inlineStr"/>
-      <c r="G481" s="2" t="inlineStr"/>
-      <c r="H481" s="2" t="inlineStr"/>
-      <c r="I481" s="2" t="inlineStr"/>
-      <c r="J481" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F481" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G481" s="2" t="inlineStr">
+        <is>
+          <t>B10-G022</t>
+        </is>
+      </c>
+      <c r="H481" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I481" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J481" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K481" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted_not_section_32</t>
         </is>
       </c>
       <c r="L481" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Assignment of leases; visible tracts are outside Section 32.</t>
         </is>
       </c>
     </row>
@@ -28731,27 +29331,47 @@
       </c>
       <c r="D482" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E482" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F482" s="2" t="inlineStr"/>
-      <c r="G482" s="2" t="inlineStr"/>
-      <c r="H482" s="2" t="inlineStr"/>
-      <c r="I482" s="2" t="inlineStr"/>
-      <c r="J482" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F482" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G482" s="2" t="inlineStr">
+        <is>
+          <t>B10-G022</t>
+        </is>
+      </c>
+      <c r="H482" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I482" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J482" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K482" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted_not_section_32</t>
         </is>
       </c>
       <c r="L482" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Corporate acknowledgment and recording continuation of 0480.</t>
         </is>
       </c>
     </row>
@@ -28771,27 +29391,47 @@
       </c>
       <c r="D483" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E483" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F483" s="2" t="inlineStr"/>
-      <c r="G483" s="2" t="inlineStr"/>
-      <c r="H483" s="2" t="inlineStr"/>
-      <c r="I483" s="2" t="inlineStr"/>
-      <c r="J483" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F483" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G483" s="2" t="inlineStr">
+        <is>
+          <t>B10-G023</t>
+        </is>
+      </c>
+      <c r="H483" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I483" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J483" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K483" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L483" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Assignment of leases first schedule page; Section 32 lease calls inspected.</t>
         </is>
       </c>
     </row>
@@ -28811,27 +29451,47 @@
       </c>
       <c r="D484" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E484" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F484" s="2" t="inlineStr"/>
-      <c r="G484" s="2" t="inlineStr"/>
-      <c r="H484" s="2" t="inlineStr"/>
-      <c r="I484" s="2" t="inlineStr"/>
-      <c r="J484" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F484" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G484" s="2" t="inlineStr">
+        <is>
+          <t>B10-G023</t>
+        </is>
+      </c>
+      <c r="H484" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I484" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J484" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K484" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L484" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Lease schedule continuation; additional Section 32 calls inspected.</t>
         </is>
       </c>
     </row>
@@ -28851,27 +29511,47 @@
       </c>
       <c r="D485" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E485" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F485" s="2" t="inlineStr"/>
-      <c r="G485" s="2" t="inlineStr"/>
-      <c r="H485" s="2" t="inlineStr"/>
-      <c r="I485" s="2" t="inlineStr"/>
-      <c r="J485" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F485" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G485" s="2" t="inlineStr">
+        <is>
+          <t>B10-G023</t>
+        </is>
+      </c>
+      <c r="H485" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I485" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J485" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K485" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L485" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Final schedule, execution, acknowledgment, and recording continuation of 0482.</t>
         </is>
       </c>
     </row>
@@ -28891,27 +29571,47 @@
       </c>
       <c r="D486" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E486" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F486" s="2" t="inlineStr"/>
-      <c r="G486" s="2" t="inlineStr"/>
-      <c r="H486" s="2" t="inlineStr"/>
-      <c r="I486" s="2" t="inlineStr"/>
-      <c r="J486" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F486" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G486" s="2" t="inlineStr">
+        <is>
+          <t>B10-G024</t>
+        </is>
+      </c>
+      <c r="H486" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I486" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J486" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K486" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L486" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Agreement of dissolution first page; partnership assets and Section 32 interest inspected.</t>
         </is>
       </c>
     </row>
@@ -28931,27 +29631,47 @@
       </c>
       <c r="D487" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E487" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F487" s="2" t="inlineStr"/>
-      <c r="G487" s="2" t="inlineStr"/>
-      <c r="H487" s="2" t="inlineStr"/>
-      <c r="I487" s="2" t="inlineStr"/>
-      <c r="J487" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F487" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G487" s="2" t="inlineStr">
+        <is>
+          <t>B10-G024</t>
+        </is>
+      </c>
+      <c r="H487" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I487" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J487" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K487" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L487" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Asset schedule continuation, allocation, signatures, acknowledgment, and recording stamp inspected.</t>
         </is>
       </c>
     </row>
@@ -28971,27 +29691,47 @@
       </c>
       <c r="D488" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E488" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F488" s="2" t="inlineStr"/>
-      <c r="G488" s="2" t="inlineStr"/>
-      <c r="H488" s="2" t="inlineStr"/>
-      <c r="I488" s="2" t="inlineStr"/>
-      <c r="J488" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F488" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G488" s="2" t="inlineStr">
+        <is>
+          <t>B10-G025</t>
+        </is>
+      </c>
+      <c r="H488" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I488" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J488" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K488" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L488" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Pipeline right-of-way; dimensions, legal, signatures, acknowledgment, and stamp inspected.</t>
         </is>
       </c>
     </row>
@@ -29011,27 +29751,47 @@
       </c>
       <c r="D489" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E489" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F489" s="2" t="inlineStr"/>
-      <c r="G489" s="2" t="inlineStr"/>
-      <c r="H489" s="2" t="inlineStr"/>
-      <c r="I489" s="2" t="inlineStr"/>
-      <c r="J489" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F489" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G489" s="2" t="inlineStr">
+        <is>
+          <t>B10-G026</t>
+        </is>
+      </c>
+      <c r="H489" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I489" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J489" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K489" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L489" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Warranty deed; mineral exceptions/reservations and retained rents inspected.</t>
         </is>
       </c>
     </row>
@@ -29051,27 +29811,47 @@
       </c>
       <c r="D490" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E490" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F490" s="2" t="inlineStr"/>
-      <c r="G490" s="2" t="inlineStr"/>
-      <c r="H490" s="2" t="inlineStr"/>
-      <c r="I490" s="2" t="inlineStr"/>
-      <c r="J490" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F490" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G490" s="2" t="inlineStr">
+        <is>
+          <t>B10-G027</t>
+        </is>
+      </c>
+      <c r="H490" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I490" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J490" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K490" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L490" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Mineral deed to L. H. Maddoux; execution, acknowledgment, and recording stamp inspected.</t>
         </is>
       </c>
     </row>
@@ -29091,27 +29871,47 @@
       </c>
       <c r="D491" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E491" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F491" s="2" t="inlineStr"/>
-      <c r="G491" s="2" t="inlineStr"/>
-      <c r="H491" s="2" t="inlineStr"/>
-      <c r="I491" s="2" t="inlineStr"/>
-      <c r="J491" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F491" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G491" s="2" t="inlineStr">
+        <is>
+          <t>B10-G028</t>
+        </is>
+      </c>
+      <c r="H491" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I491" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J491" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K491" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L491" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Separate mineral deed to A. E. Maddoux; execution, acknowledgment, and recording stamp inspected.</t>
         </is>
       </c>
     </row>
@@ -29131,27 +29931,47 @@
       </c>
       <c r="D492" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E492" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F492" s="2" t="inlineStr"/>
-      <c r="G492" s="2" t="inlineStr"/>
-      <c r="H492" s="2" t="inlineStr"/>
-      <c r="I492" s="2" t="inlineStr"/>
-      <c r="J492" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F492" s="2" t="inlineStr">
+        <is>
+          <t>poor-negative</t>
+        </is>
+      </c>
+      <c r="G492" s="2" t="inlineStr">
+        <is>
+          <t>B10-G029</t>
+        </is>
+      </c>
+      <c r="H492" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I492" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J492" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K492" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted_with_assumption</t>
         </is>
       </c>
       <c r="L492" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Negative image inverted, channel-separated, enlarged, and cropped; parties, $12,500 debt, and S/2 SW/4 plus W/2 SE/4 legal recovered. Recording data is not visible.</t>
         </is>
       </c>
     </row>
@@ -29171,27 +29991,47 @@
       </c>
       <c r="D493" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E493" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F493" s="2" t="inlineStr"/>
-      <c r="G493" s="2" t="inlineStr"/>
-      <c r="H493" s="2" t="inlineStr"/>
-      <c r="I493" s="2" t="inlineStr"/>
-      <c r="J493" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F493" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G493" s="2" t="inlineStr">
+        <is>
+          <t>B10-G030</t>
+        </is>
+      </c>
+      <c r="H493" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I493" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J493" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K493" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L493" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Mineral deed; five-acre interest, signature, acknowledgment, and stamp inspected.</t>
         </is>
       </c>
     </row>
@@ -29211,27 +30051,47 @@
       </c>
       <c r="D494" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E494" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F494" s="2" t="inlineStr"/>
-      <c r="G494" s="2" t="inlineStr"/>
-      <c r="H494" s="2" t="inlineStr"/>
-      <c r="I494" s="2" t="inlineStr"/>
-      <c r="J494" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F494" s="2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="G494" s="2" t="inlineStr">
+        <is>
+          <t>B10-G031</t>
+        </is>
+      </c>
+      <c r="H494" s="2" t="inlineStr">
+        <is>
+          <t>first_or_single_page</t>
+        </is>
+      </c>
+      <c r="I494" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J494" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K494" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="L494" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Mineral deed returning five-acre interest; capacities, signatures, acknowledgment, and stamp inspected.</t>
         </is>
       </c>
     </row>
@@ -29251,27 +30111,47 @@
       </c>
       <c r="D495" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E495" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F495" s="2" t="inlineStr"/>
-      <c r="G495" s="2" t="inlineStr"/>
-      <c r="H495" s="2" t="inlineStr"/>
-      <c r="I495" s="2" t="inlineStr"/>
-      <c r="J495" s="2" t="inlineStr"/>
+          <t>reviewed_instrument_page</t>
+        </is>
+      </c>
+      <c r="F495" s="2" t="inlineStr">
+        <is>
+          <t>fair-negative</t>
+        </is>
+      </c>
+      <c r="G495" s="2" t="inlineStr">
+        <is>
+          <t>B10-G032</t>
+        </is>
+      </c>
+      <c r="H495" s="2" t="inlineStr">
+        <is>
+          <t>first_page</t>
+        </is>
+      </c>
+      <c r="I495" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J495" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K495" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_boundary_instrument</t>
         </is>
       </c>
       <c r="L495" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Cover of Seventh Supplemental Indenture; recording stamps and handwritten marginal references inspected.</t>
         </is>
       </c>
     </row>
@@ -29291,27 +30171,47 @@
       </c>
       <c r="D496" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E496" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F496" s="2" t="inlineStr"/>
-      <c r="G496" s="2" t="inlineStr"/>
-      <c r="H496" s="2" t="inlineStr"/>
-      <c r="I496" s="2" t="inlineStr"/>
-      <c r="J496" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F496" s="2" t="inlineStr">
+        <is>
+          <t>fair-negative</t>
+        </is>
+      </c>
+      <c r="G496" s="2" t="inlineStr">
+        <is>
+          <t>B10-G032</t>
+        </is>
+      </c>
+      <c r="H496" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I496" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J496" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K496" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_boundary_instrument</t>
         </is>
       </c>
       <c r="L496" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Indenture page 1; parties and recitals inspected.</t>
         </is>
       </c>
     </row>
@@ -29331,27 +30231,47 @@
       </c>
       <c r="D497" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E497" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F497" s="2" t="inlineStr"/>
-      <c r="G497" s="2" t="inlineStr"/>
-      <c r="H497" s="2" t="inlineStr"/>
-      <c r="I497" s="2" t="inlineStr"/>
-      <c r="J497" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F497" s="2" t="inlineStr">
+        <is>
+          <t>fair-negative</t>
+        </is>
+      </c>
+      <c r="G497" s="2" t="inlineStr">
+        <is>
+          <t>B10-G032</t>
+        </is>
+      </c>
+      <c r="H497" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I497" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J497" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K497" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_boundary_instrument</t>
         </is>
       </c>
       <c r="L497" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Indenture pages 2-3 photographed as spread; recitals inspected.</t>
         </is>
       </c>
     </row>
@@ -29371,27 +30291,47 @@
       </c>
       <c r="D498" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E498" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F498" s="2" t="inlineStr"/>
-      <c r="G498" s="2" t="inlineStr"/>
-      <c r="H498" s="2" t="inlineStr"/>
-      <c r="I498" s="2" t="inlineStr"/>
-      <c r="J498" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F498" s="2" t="inlineStr">
+        <is>
+          <t>fair-negative</t>
+        </is>
+      </c>
+      <c r="G498" s="2" t="inlineStr">
+        <is>
+          <t>B10-G032</t>
+        </is>
+      </c>
+      <c r="H498" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I498" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J498" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K498" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_boundary_instrument</t>
         </is>
       </c>
       <c r="L498" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Indenture pages 4-5 photographed as spread; Series E bond terms inspected.</t>
         </is>
       </c>
     </row>
@@ -29411,27 +30351,47 @@
       </c>
       <c r="D499" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E499" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F499" s="2" t="inlineStr"/>
-      <c r="G499" s="2" t="inlineStr"/>
-      <c r="H499" s="2" t="inlineStr"/>
-      <c r="I499" s="2" t="inlineStr"/>
-      <c r="J499" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F499" s="2" t="inlineStr">
+        <is>
+          <t>fair-negative</t>
+        </is>
+      </c>
+      <c r="G499" s="2" t="inlineStr">
+        <is>
+          <t>B10-G032</t>
+        </is>
+      </c>
+      <c r="H499" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I499" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J499" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K499" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_boundary_instrument</t>
         </is>
       </c>
       <c r="L499" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Indenture pages 6-7 photographed as spread; redemption and sinking-fund terms inspected.</t>
         </is>
       </c>
     </row>
@@ -29451,27 +30411,47 @@
       </c>
       <c r="D500" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E500" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F500" s="2" t="inlineStr"/>
-      <c r="G500" s="2" t="inlineStr"/>
-      <c r="H500" s="2" t="inlineStr"/>
-      <c r="I500" s="2" t="inlineStr"/>
-      <c r="J500" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F500" s="2" t="inlineStr">
+        <is>
+          <t>fair-negative</t>
+        </is>
+      </c>
+      <c r="G500" s="2" t="inlineStr">
+        <is>
+          <t>B10-G032</t>
+        </is>
+      </c>
+      <c r="H500" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I500" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J500" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K500" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_boundary_instrument</t>
         </is>
       </c>
       <c r="L500" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Indenture pages 8-9 photographed as spread; sinking-fund provisions inspected.</t>
         </is>
       </c>
     </row>
@@ -29491,27 +30471,47 @@
       </c>
       <c r="D501" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="E501" s="2" t="inlineStr">
         <is>
-          <t>INVENTORIED — NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="F501" s="2" t="inlineStr"/>
-      <c r="G501" s="2" t="inlineStr"/>
-      <c r="H501" s="2" t="inlineStr"/>
-      <c r="I501" s="2" t="inlineStr"/>
-      <c r="J501" s="2" t="inlineStr"/>
+          <t>continuation_or_mixed_page</t>
+        </is>
+      </c>
+      <c r="F501" s="2" t="inlineStr">
+        <is>
+          <t>fair-negative</t>
+        </is>
+      </c>
+      <c r="G501" s="2" t="inlineStr">
+        <is>
+          <t>B10-G032</t>
+        </is>
+      </c>
+      <c r="H501" s="2" t="inlineStr">
+        <is>
+          <t>continuation</t>
+        </is>
+      </c>
+      <c r="I501" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J501" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
       <c r="K501" s="2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>partial_boundary_instrument</t>
         </is>
       </c>
       <c r="L501" s="2" t="inlineStr">
         <is>
-          <t>Natural filename order; Drive file ID preserved before interpretation.</t>
+          <t>Indenture pages 10-11 photographed as spread; bond form inspected. Text plainly continues past the scoped boundary.</t>
         </is>
       </c>
     </row>

</xml_diff>